<commit_message>
Expand interview prep workbook content
Co-authored-by: impalalogis <impalalogis@gmail.com>
</commit_message>
<xml_diff>
--- a/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
+++ b/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1311,1114 +1311,307 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SQL Basics</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SELECT / WHERE / ORDER BY basics</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>- Core query structure with filtering and sorting.
+SQL:
+```
+SELECT col1, col2
+FROM table_name
+WHERE col1 &gt; 10
+ORDER BY col2 DESC;
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SQL Filtering</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>LIKE, IN, BETWEEN, IS NULL filters</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>- Common predicates for filtering rows.
+SQL:
+```
+SELECT name
+FROM city
+WHERE name LIKE 'P%'
+  AND country_id IN (1, 2)
+  AND population BETWEEN 500000 AND 5000000
+  AND rating IS NOT NULL;
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>SQL Joins</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>INNER vs LEFT vs RIGHT vs FULL vs CROSS</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>- INNER returns matches, LEFT/RIGHT keep all rows from one side, FULL keeps all rows, CROSS returns all combinations.
+SQL:
+```
+SELECT c.name, co.name
+FROM city c
+LEFT JOIN country co ON c.country_id = co.id;
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SQL Aggregation</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>GROUP BY and HAVING</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>- GROUP BY aggregates by key; HAVING filters aggregates.
+SQL:
+```
+SELECT country_id, AVG(rating) AS avg_rating
+FROM city
+GROUP BY country_id
+HAVING AVG(rating) &gt; 3;
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SQL Aggregation</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Aggregate functions (COUNT, SUM, AVG, MIN, MAX)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>- Summarize numeric values per group or whole table.
+SQL:
+```
+SELECT COUNT(*) AS total, MIN(population) AS min_pop, MAX(population) AS max_pop
+FROM country;
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SQL Subqueries</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Single-value and multi-value subqueries</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>- Use scalar subqueries with operators and multi-row subqueries with IN/EXISTS.
+SQL:
+```
+SELECT name
+FROM city
+WHERE rating = (SELECT rating FROM city WHERE name = 'Paris');
+SELECT name
+FROM city
+WHERE country_id IN (SELECT id FROM country WHERE population &gt; 20000000);
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SQL Subqueries</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Correlated subquery</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>- Subquery references the outer query for row-by-row evaluation.
+SQL:
+```
+SELECT *
+FROM city c
+WHERE population &gt; (
+  SELECT AVG(population)
+  FROM city c2
+  WHERE c2.country_id = c.country_id
+);
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SQL Set Operations</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>UNION / INTERSECT / EXCEPT</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>- Combine result sets with set operations.
+SQL:
+```
+SELECT name FROM cycling WHERE country = 'DE'
+UNION
+SELECT name FROM skating WHERE country = 'DE';
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SQL Functions</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>String functions (CONCAT, LOWER/UPPER, LENGTH, SUBSTRING, REPLACE)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>- Useful text transformations.
+SQL:
+```
+SELECT CONCAT(first_name, ' ', last_name) AS full_name,
+       LOWER(email) AS email_lc,
+       LENGTH(name) AS name_len,
+       SUBSTRING(name, 1, 3) AS prefix,
+       REPLACE(name, ' ', '_') AS name_key
+FROM users;
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SQL Functions</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Numeric functions and CAST</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>- Numeric utilities and type conversion.
+SQL:
+```
+SELECT ROUND(price, 2) AS price_round,
+       CEIL(discount) AS disc_ceil,
+       FLOOR(discount) AS disc_floor,
+       ABS(delta) AS abs_delta,
+       CAST(amount AS DECIMAL(10,2)) AS amt
+FROM sales;
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SQL NULLs</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>COALESCE, NULLIF, CASE WHEN</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>- Handle missing values and conditional logic.
+SQL:
+```
+SELECT COALESCE(city, 'Unknown') AS city,
+       NULLIF(last_month, 0) AS last_month_safe,
+       CASE WHEN score &gt;= 90 THEN 'A' ELSE 'B' END AS grade
+FROM results;
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SQL Date/Time</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>CURRENT_DATE, INTERVAL, EXTRACT, AT TIME ZONE</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>- Work with dates, timestamps, and time zones.
+SQL:
+```
+SELECT CURRENT_DATE AS today,
+       order_date + INTERVAL '7' DAY AS next_week,
+       EXTRACT(YEAR FROM order_date) AS order_year
+FROM orders;
+```</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>OLTP vs OLAP</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>- OLTP: transactional, normalized schema, many small writes, current data.
-- OLAP: analytical, denormalized schema, read-heavy, historical data.
-- OLAP favors complex queries and aggregates; OLTP favors fast inserts/updates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>ACID properties</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>- Atomicity: all or nothing.
-- Consistency: transactions move DB between valid states.
-- Isolation: concurrent transactions behave as if serial.
-- Durability: committed data survives failures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Schema-on-Read vs Schema-on-Write</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>- Schema-on-Write: enforce schema before data is stored (DWH, RDBMS).
-- Schema-on-Read: apply schema when data is read (data lakes).
-- Trade-off: upfront governance vs flexibility.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Data Warehouse vs Data Mart vs Data Lake vs Data Mesh</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>- Data Warehouse: centralized, curated, structured analytics store.
-- Data Mart: department or subject-specific subset of a warehouse.
-- Data Lake: raw, multi-format storage with schema-on-read.
-- Data Mesh: decentralized domain-owned data products with shared governance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>ETL vs ELT</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>- ETL: transform before loading; good for controlled environments.
-- ELT: load raw data, transform in the target system; good for scalable cloud DWH.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Star Schema vs Snowflake Schema</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>- Star: denormalized dimensions, simpler joins, faster queries.
-- Snowflake: normalized dimensions, less redundancy, more joins.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Fact vs Dimension Tables</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>- Fact: measures and foreign keys (e.g., sales_amount, qty).
-- Dimension: descriptive attributes (e.g., customer, product, date).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>SCD Types 0,1,2,3,4,6</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>- Type 0: no changes stored (retain original).
-- Type 1: overwrite old value.
-- Type 2: add new row with effective dates, keep history.
-- Type 3: add new column for previous value (limited history).
-- Type 4: separate history table.
-- Type 6: hybrid (1+2+3) with current and history columns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>DWH Keys</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>- Primary: unique identifier in table.
-- Surrogate: system-generated key (no business meaning).
-- Natural: business key from source.
-- Composite: multiple columns form key.
-- Candidate: potential primary key.
-- Alternate: candidate key not chosen as primary.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>MERGE/UPSERT logic</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>- Match on business key, update if exists, insert if not.
-SQL:
-```
-MERGE INTO dim_customer AS t
-USING staging_customer AS s
-ON t.customer_id = s.customer_id
-WHEN MATCHED THEN
-  UPDATE SET t.name = s.name, t.city = s.city, t.updated_at = CURRENT_TIMESTAMP
-WHEN NOT MATCHED THEN
-  INSERT (customer_id, name, city, created_at)
-  VALUES (s.customer_id, s.name, s.city, CURRENT_TIMESTAMP);
-```</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Shallow copy vs deep copy</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>- Shallow copy copies the outer container; nested objects are shared.
-- Deep copy recursively copies nested objects.
-Example:
-```
-import copy
-x = [[1, 2], [3, 4]]
-sh = copy.copy(x)
-dp = copy.deepcopy(x)
-sh[0].append(99)
-# x changes, dp does not
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Multithreading in Python</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>- Use threading for IO-bound tasks; GIL limits CPU-bound parallelism.
-Example:
-```
-from threading import Thread
-def fetch(url):
-    ...
-threads = [Thread(target=fetch, args=(u,)) for u in urls]
-[t.start() for t in threads]
-[t.join() for t in threads]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Django architecture</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>- Django follows MTV: Model (ORM), Template (UI), View (request logic).
-- URL dispatcher and middleware connect requests to views.
-Example:
-```
-# urls.py
-path('users/', views.user_list)
-# views.py
-return render(request, 'users.html', {'users': User.objects.all()})
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Pickling vs unpickling</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>- Pickling serializes objects to bytes; unpickling restores them.
-Example:
-```
-import pickle
-blob = pickle.dumps({'a': 1})
-obj = pickle.loads(blob)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Memory management in Python</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>- Uses reference counting plus cyclic GC; small objects use pymalloc arenas.
-Example:
-```
-import gc
-obj = []
-obj.append(obj)
-del obj
-gc.collect()
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Pass-by-reference vs pass-by-value</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>- Python passes object references (call-by-object).
-- Mutating a passed mutable affects the caller; rebinding does not.
-Example:
-```
-def f(lst):
-    lst.append(1)
-a = []
-f(a)  # a becomes [1]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Random number generation</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>- Use random for general RNG, seed for reproducibility; use secrets for crypto.
-Example:
-```
-import random
-random.seed(42)
-random.randint(1, 10)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>// operator</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>- Floor division; result is the floor of true division.
-Example:
-```
-7 // 3   # 2
--7 // 3  # -3
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>"is" operator</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>- Checks object identity, not equality.
-Example:
-```
-a = [1]
-b = [1]
-(a == b)  # True
-(a is b)  # False
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>pass statement</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>- No-op placeholder used where syntax requires a statement.
-Example:
-```
-def todo():
-    pass
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Check if string is alphanumeric</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>- Use str.isalnum().
-Example:
-```
-'sku123'.isalnum()  # True
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Merge elements in sequences</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>- Concatenate or chain sequences; zip to pair elements.
-Example:
-```
-import itertools
-merged = list(itertools.chain([1, 2], [3, 4]))
-paired = list(zip([1, 2], ['a', 'b']))
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Remove leading whitespace</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>- Use lstrip().
-Example:
-```
-'  abc'.lstrip()  # 'abc'
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>replace() usage</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>- Replace substrings with str.replace(old, new, count).
-Example:
-```
-'2026-01-26'.replace('-', '/')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>del vs remove()</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>- del deletes by index or deletes a name; remove deletes first matching value.
-Example:
-```
-a = [1, 2, 3]
-del a[0]    # [2, 3]
-a.remove(3) # [2]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>append() vs extend()</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>- append adds one object; extend adds elements from an iterable.
-Example:
-```
-a = [1]
-a.append([2, 3])  # [1, [2, 3]]
-a.extend([4, 5])  # [1, [2, 3], 4, 5]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Reverse file contents</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>- Read lines and write/print in reverse order.
-Example:
-```
-with open('f.txt') as f:
-    lines = f.readlines()
-rev = ''.join(reversed(lines))
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>List vs Tuple</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>- List is mutable; tuple is immutable and can be hashable.
-Example:
-```
-coords = (10, 20)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Docstring</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>- First string literal in a module/class/function; available via __doc__.
-Example:
-```
-def add(a, b):
-    'Return sum of a and b.'
-    return a + b
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>split() function</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>- str.split(sep, maxsplit) splits a string into a list.
-Example:
-```
-'foo,bar'.split(',')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>*args and **kwargs</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>- *args collects positional args; **kwargs collects keyword args.
-Example:
-```
-def f(*args, **kwargs):
-    return args, kwargs
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>First-class functions</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>- Functions can be assigned, passed, and returned like data.
-Example:
-```
-def apply(f, x):
-    return f(x)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>What is __name__</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>- Module name; when run directly, __name__ == '__main__'.
-Example:
-```
-if __name__ == '__main__':
-    main()
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>NumPy arrays</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>- N-dimensional, homogeneous arrays with vectorized operations.
-Example:
-```
-import numpy as np
-arr = np.array([1, 2, 3])
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Matrices vs arrays</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>- Arrays are general n-D; matrices are strictly 2-D. Prefer arrays with @.
-Example:
-```
-A = np.array([[1, 2], [3, 4]])
-B = np.array([[5, 6], [7, 8]])
-A @ B
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>argsort usage</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>- Returns indices that would sort an array.
-Example:
-```
-import numpy as np
-x = np.array([30, 10, 20])
-idx = np.argsort(x)  # [1, 2, 0]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>vstack usage</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>- Stack arrays vertically (row-wise).
-Example:
-```
-import numpy as np
-np.vstack([[1, 2], [3, 4]])
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>DecisionTree import</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>- Import from sklearn.tree.
-Example:
-```
-from sklearn.tree import DecisionTreeClassifier
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Pandas read_csv encoding issue</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>- Specify encoding and error handling.
-Example:
-```
-import pandas as pd
-df = pd.read_csv('data.csv', encoding='latin1', errors='replace')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Matplotlib linewidth</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>- Use linewidth (or lw) in plotting calls.
-Example:
-```
-import matplotlib.pyplot as plt
-plt.plot(x, y, linewidth=2)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>reindex vs reset_index</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>- reindex changes index labels/ordering; reset_index moves index to a column.
-Example:
-```
-df = df.reindex(['b', 'a'])
-df = df.reset_index(drop=True)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>xrange vs range</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>- Python2: xrange is lazy, range builds list. Python3: range is lazy; xrange removed.
-Example:
-```
-for i in range(3):
-    print(i)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Check if DataFrame is empty</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>- Use df.empty (True if no rows or columns).
-Example:
-```
-df.empty
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Sort array by column</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>- Use argsort on the target column.
-Example:
-```
-import numpy as np
-arr = np.array([[3, 1], [2, 9], [1, 5]])
-arr[arr[:, 0].argsort()]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Create Series from list/array/dict</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>- Use pd.Series with different inputs.
-Example:
-```
-import pandas as pd
-pd.Series([1, 2])
-pd.Series({'a': 1, 'b': 2})
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Items not common between two Series</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>- Use symmetric difference with isin.
-Example:
-```
-import pandas as pd
-s1 = pd.Series([1, 2, 3])
-s2 = pd.Series([2, 3, 4])
-not_common = pd.concat([s1[~s1.isin(s2)], s2[~s2.isin(s1)]])
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Replace all except top 2 frequent values</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>- Keep top 2 values, replace others.
-Example:
-```
-import pandas as pd
-s = pd.Series(['a', 'b', 'a', 'c', 'd', 'a', 'b'])
-top2 = s.value_counts().nlargest(2).index
-s2 = s.where(s.isin(top2), other='Other')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Find multiples of 3 in Series</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>- Filter using modulo.
-Example:
-```
-import pandas as pd
-s = pd.Series([1, 3, 4, 6])
-mult3 = s[s % 3 == 0]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Euclidean distance between Series</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>- Compute norm of the difference.
-Example:
-```
-import numpy as np
-import pandas as pd
-s1 = pd.Series([1, 2, 3])
-s2 = pd.Series([4, 5, 6])
-dist = np.linalg.norm(s1 - s2)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Reverse DataFrame rows</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>- Reverse with iloc and reset index.
-Example:
-```
-df_rev = df.iloc[::-1].reset_index(drop=True)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Overfitting with train/test split</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>- Overfitting shows strong train but weak test performance.
-- Mitigate with validation, cross-validation, regularization, and simpler models.
-Example:
-```
-from sklearn.model_selection import train_test_split
-X_train, X_test, y_train, y_test = train_test_split(X, y, test_size=0.2, random_state=42)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Seaborn usage</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>- High-level statistical plotting built on matplotlib.
-Example:
-```
-import seaborn as sns
-sns.barplot(data=df, x='dept', y='salary')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Python literals</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>- Fixed values in source code: numbers, strings, bytes, booleans, None, collections.
-Example:
-```
-42, 3.14, 'text', b'bin', True, None, [1, 2], {'a': 1}
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Decorators</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>- Functions that wrap other functions to add behavior.
-Example:
-```
-def log_call(f):
-    def wrapper(*args, **kwargs):
-        print(f.__name__)
-        return f(*args, **kwargs)
-    return wrapper
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Slicing</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>- Use start:stop:step; stop is exclusive.
-Example:
-```
-arr = [0, 1, 2, 3, 4]
-arr[1:4:2]  # [1, 3]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Keywords in Python</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>- Reserved words that cannot be identifiers; see keyword.kwlist.
-Example:
-```
-import keyword
-keyword.kwlist
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Lambda functions</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>- Anonymous, single-expression functions.
-Example:
-```
-add = lambda x, y: x + y
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>continue vs break vs pass</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>- continue skips to next iteration; break exits loop; pass does nothing.
-Example:
-```
-for i in range(3):
-    if i == 1:
-        continue
-    if i == 2:
-        break
-    pass
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Iterators</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>- Iterators implement __iter__ and __next__; use iter() and next().
-Example:
-```
-it = iter([1, 2, 3])
-next(it)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Python namespaces</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>- Namespaces map names to objects; scope order is LEGB.
-Example:
-```
-x = 1
-def f():
-    x = 2  # local
-```</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2446,6 +1639,1489 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>OLTP vs OLAP</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>- OLTP: transactional, normalized schema, many small writes, current data.
+- OLAP: analytical, denormalized schema, read-heavy, historical data.
+- OLAP favors complex queries and aggregates; OLTP favors fast inserts/updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ACID properties</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>- Atomicity: all or nothing.
+- Consistency: transactions move DB between valid states.
+- Isolation: concurrent transactions behave as if serial.
+- Durability: committed data survives failures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Schema-on-Read vs Schema-on-Write</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>- Schema-on-Write: enforce schema before data is stored (DWH, RDBMS).
+- Schema-on-Read: apply schema when data is read (data lakes).
+- Trade-off: upfront governance vs flexibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Data Warehouse vs Data Mart vs Data Lake vs Data Mesh</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>- Data Warehouse: centralized, curated, structured analytics store.
+- Data Mart: department or subject-specific subset of a warehouse.
+- Data Lake: raw, multi-format storage with schema-on-read.
+- Data Mesh: decentralized domain-owned data products with shared governance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ETL vs ELT</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>- ETL: transform before loading; good for controlled environments.
+- ELT: load raw data, transform in the target system; good for scalable cloud DWH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Star Schema vs Snowflake Schema</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>- Star: denormalized dimensions, simpler joins, faster queries.
+- Snowflake: normalized dimensions, less redundancy, more joins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Fact vs Dimension Tables</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>- Fact: measures and foreign keys (e.g., sales_amount, qty).
+- Dimension: descriptive attributes (e.g., customer, product, date).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SCD Types 0,1,2,3,4,6</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>- Type 0: no changes stored (retain original).
+- Type 1: overwrite old value.
+- Type 2: add new row with effective dates, keep history.
+- Type 3: add new column for previous value (limited history).
+- Type 4: separate history table.
+- Type 6: hybrid (1+2+3) with current and history columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>DWH Keys</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>- Primary: unique identifier in table.
+- Surrogate: system-generated key (no business meaning).
+- Natural: business key from source.
+- Composite: multiple columns form key.
+- Candidate: potential primary key.
+- Alternate: candidate key not chosen as primary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>MERGE/UPSERT logic</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>- Match on business key, update if exists, insert if not.
+SQL:
+```
+MERGE INTO dim_customer AS t
+USING staging_customer AS s
+ON t.customer_id = s.customer_id
+WHEN MATCHED THEN
+  UPDATE SET t.name = s.name, t.city = s.city, t.updated_at = CURRENT_TIMESTAMP
+WHEN NOT MATCHED THEN
+  INSERT (customer_id, name, city, created_at)
+  VALUES (s.customer_id, s.name, s.city, CURRENT_TIMESTAMP);
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Data modeling types (conceptual, logical, physical)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>- Conceptual: high-level business entities and relationships.
+- Logical: detailed entities, attributes, and relationships.
+- Physical: storage details like indexes, partitions, and data types.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Galaxy schema (fact constellation)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>- Multiple fact tables share common dimension tables.
+- Useful for complex warehouses with related business processes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Normalized vs denormalized models</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>- Normalized: reduces redundancy, improves integrity, more joins.
+- Denormalized: faster reads, simpler queries, more storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Fact table grain</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>- Grain defines the level of detail per fact row (e.g., per order line, per day).
+- Set grain before adding dimensions/measures to avoid ambiguity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Data modeling best practices</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>- Align with business requirements and reporting needs.
+- Design for data quality and consistent definitions.
+- Balance normalization vs performance.
+- Plan for scalability and document the model.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Shallow copy vs deep copy</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>- Shallow copy copies the outer container; nested objects are shared.
+- Deep copy recursively copies nested objects.
+Example:
+```
+import copy
+x = [[1, 2], [3, 4]]
+sh = copy.copy(x)
+dp = copy.deepcopy(x)
+sh[0].append(99)
+# x changes, dp does not
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Multithreading in Python</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>- Use threading for IO-bound tasks; GIL limits CPU-bound parallelism.
+Example:
+```
+from threading import Thread
+def fetch(url):
+    ...
+threads = [Thread(target=fetch, args=(u,)) for u in urls]
+[t.start() for t in threads]
+[t.join() for t in threads]
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Django architecture</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>- Django follows MTV: Model (ORM), Template (UI), View (request logic).
+- URL dispatcher and middleware connect requests to views.
+Example:
+```
+# urls.py
+path('users/', views.user_list)
+# views.py
+return render(request, 'users.html', {'users': User.objects.all()})
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Pickling vs unpickling</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>- Pickling serializes objects to bytes; unpickling restores them.
+Example:
+```
+import pickle
+blob = pickle.dumps({'a': 1})
+obj = pickle.loads(blob)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Memory management in Python</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>- Uses reference counting plus cyclic GC; small objects use pymalloc arenas.
+Example:
+```
+import gc
+obj = []
+obj.append(obj)
+del obj
+gc.collect()
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Pass-by-reference vs pass-by-value</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>- Python passes object references (call-by-object).
+- Mutating a passed mutable affects the caller; rebinding does not.
+Example:
+```
+def f(lst):
+    lst.append(1)
+a = []
+f(a)  # a becomes [1]
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Random number generation</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>- Use random for general RNG, seed for reproducibility; use secrets for crypto.
+Example:
+```
+import random
+random.seed(42)
+random.randint(1, 10)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>// operator</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>- Floor division; result is the floor of true division.
+Example:
+```
+7 // 3   # 2
+-7 // 3  # -3
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>"is" operator</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>- Checks object identity, not equality.
+Example:
+```
+a = [1]
+b = [1]
+(a == b)  # True
+(a is b)  # False
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>pass statement</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>- No-op placeholder used where syntax requires a statement.
+Example:
+```
+def todo():
+    pass
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Check if string is alphanumeric</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>- Use str.isalnum().
+Example:
+```
+'sku123'.isalnum()  # True
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Merge elements in sequences</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>- Concatenate or chain sequences; zip to pair elements.
+Example:
+```
+import itertools
+merged = list(itertools.chain([1, 2], [3, 4]))
+paired = list(zip([1, 2], ['a', 'b']))
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Remove leading whitespace</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>- Use lstrip().
+Example:
+```
+'  abc'.lstrip()  # 'abc'
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>replace() usage</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>- Replace substrings with str.replace(old, new, count).
+Example:
+```
+'2026-01-26'.replace('-', '/')
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>del vs remove()</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>- del deletes by index or deletes a name; remove deletes first matching value.
+Example:
+```
+a = [1, 2, 3]
+del a[0]    # [2, 3]
+a.remove(3) # [2]
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>append() vs extend()</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>- append adds one object; extend adds elements from an iterable.
+Example:
+```
+a = [1]
+a.append([2, 3])  # [1, [2, 3]]
+a.extend([4, 5])  # [1, [2, 3], 4, 5]
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Reverse file contents</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>- Read lines and write/print in reverse order.
+Example:
+```
+with open('f.txt') as f:
+    lines = f.readlines()
+rev = ''.join(reversed(lines))
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>List vs Tuple</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>- List is mutable; tuple is immutable and can be hashable.
+Example:
+```
+coords = (10, 20)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Docstring</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>- First string literal in a module/class/function; available via __doc__.
+Example:
+```
+def add(a, b):
+    'Return sum of a and b.'
+    return a + b
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>split() function</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>- str.split(sep, maxsplit) splits a string into a list.
+Example:
+```
+'foo,bar'.split(',')
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>*args and **kwargs</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>- *args collects positional args; **kwargs collects keyword args.
+Example:
+```
+def f(*args, **kwargs):
+    return args, kwargs
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>First-class functions</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>- Functions can be assigned, passed, and returned like data.
+Example:
+```
+def apply(f, x):
+    return f(x)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>What is __name__</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>- Module name; when run directly, __name__ == '__main__'.
+Example:
+```
+if __name__ == '__main__':
+    main()
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>NumPy arrays</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>- N-dimensional, homogeneous arrays with vectorized operations.
+Example:
+```
+import numpy as np
+arr = np.array([1, 2, 3])
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Matrices vs arrays</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>- Arrays are general n-D; matrices are strictly 2-D. Prefer arrays with @.
+Example:
+```
+A = np.array([[1, 2], [3, 4]])
+B = np.array([[5, 6], [7, 8]])
+A @ B
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>argsort usage</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>- Returns indices that would sort an array.
+Example:
+```
+import numpy as np
+x = np.array([30, 10, 20])
+idx = np.argsort(x)  # [1, 2, 0]
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>vstack usage</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>- Stack arrays vertically (row-wise).
+Example:
+```
+import numpy as np
+np.vstack([[1, 2], [3, 4]])
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>DecisionTree import</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>- Import from sklearn.tree.
+Example:
+```
+from sklearn.tree import DecisionTreeClassifier
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Pandas read_csv encoding issue</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>- Specify encoding and error handling.
+Example:
+```
+import pandas as pd
+df = pd.read_csv('data.csv', encoding='latin1', errors='replace')
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Matplotlib linewidth</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>- Use linewidth (or lw) in plotting calls.
+Example:
+```
+import matplotlib.pyplot as plt
+plt.plot(x, y, linewidth=2)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>reindex vs reset_index</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>- reindex changes index labels/ordering; reset_index moves index to a column.
+Example:
+```
+df = df.reindex(['b', 'a'])
+df = df.reset_index(drop=True)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>xrange vs range</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>- Python2: xrange is lazy, range builds list. Python3: range is lazy; xrange removed.
+Example:
+```
+for i in range(3):
+    print(i)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Check if DataFrame is empty</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>- Use df.empty (True if no rows or columns).
+Example:
+```
+df.empty
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Sort array by column</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>- Use argsort on the target column.
+Example:
+```
+import numpy as np
+arr = np.array([[3, 1], [2, 9], [1, 5]])
+arr[arr[:, 0].argsort()]
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Create Series from list/array/dict</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>- Use pd.Series with different inputs.
+Example:
+```
+import pandas as pd
+pd.Series([1, 2])
+pd.Series({'a': 1, 'b': 2})
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Items not common between two Series</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>- Use symmetric difference with isin.
+Example:
+```
+import pandas as pd
+s1 = pd.Series([1, 2, 3])
+s2 = pd.Series([2, 3, 4])
+not_common = pd.concat([s1[~s1.isin(s2)], s2[~s2.isin(s1)]])
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Replace all except top 2 frequent values</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>- Keep top 2 values, replace others.
+Example:
+```
+import pandas as pd
+s = pd.Series(['a', 'b', 'a', 'c', 'd', 'a', 'b'])
+top2 = s.value_counts().nlargest(2).index
+s2 = s.where(s.isin(top2), other='Other')
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Find multiples of 3 in Series</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>- Filter using modulo.
+Example:
+```
+import pandas as pd
+s = pd.Series([1, 3, 4, 6])
+mult3 = s[s % 3 == 0]
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Euclidean distance between Series</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>- Compute norm of the difference.
+Example:
+```
+import numpy as np
+import pandas as pd
+s1 = pd.Series([1, 2, 3])
+s2 = pd.Series([4, 5, 6])
+dist = np.linalg.norm(s1 - s2)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Reverse DataFrame rows</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>- Reverse with iloc and reset index.
+Example:
+```
+df_rev = df.iloc[::-1].reset_index(drop=True)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Overfitting with train/test split</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>- Overfitting shows strong train but weak test performance.
+- Mitigate with validation, cross-validation, regularization, and simpler models.
+Example:
+```
+from sklearn.model_selection import train_test_split
+X_train, X_test, y_train, y_test = train_test_split(X, y, test_size=0.2, random_state=42)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Seaborn usage</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>- High-level statistical plotting built on matplotlib.
+Example:
+```
+import seaborn as sns
+sns.barplot(data=df, x='dept', y='salary')
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Python literals</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>- Fixed values in source code: numbers, strings, bytes, booleans, None, collections.
+Example:
+```
+42, 3.14, 'text', b'bin', True, None, [1, 2], {'a': 1}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Decorators</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>- Functions that wrap other functions to add behavior.
+Example:
+```
+def log_call(f):
+    def wrapper(*args, **kwargs):
+        print(f.__name__)
+        return f(*args, **kwargs)
+    return wrapper
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Slicing</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>- Use start:stop:step; stop is exclusive.
+Example:
+```
+arr = [0, 1, 2, 3, 4]
+arr[1:4:2]  # [1, 3]
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Keywords in Python</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>- Reserved words that cannot be identifiers; see keyword.kwlist.
+Example:
+```
+import keyword
+keyword.kwlist
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Lambda functions</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>- Anonymous, single-expression functions.
+Example:
+```
+add = lambda x, y: x + y
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>continue vs break vs pass</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>- continue skips to next iteration; break exits loop; pass does nothing.
+Example:
+```
+for i in range(3):
+    if i == 1:
+        continue
+    if i == 2:
+        break
+    pass
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Iterators</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>- Iterators implement __iter__ and __next__; use iter() and next().
+Example:
+```
+it = iter([1, 2, 3])
+next(it)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Python namespaces</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>- Namespaces map names to objects; scope order is LEGB.
+Example:
+```
+x = 1
+def f():
+    x = 2  # local
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Python features (interpreted, dynamically typed)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>- Python is interpreted and dynamically typed; types are checked at runtime.
+- Enables rapid development and flexibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>PEP 8</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>- Python Enhancement Proposal for style and formatting.
+- Consistent naming, indentation, and readability guidelines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Global vs local variables</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>- Local variables live inside a function.
+- Global variables are defined at module scope and accessible everywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Python case sensitivity</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>- Python is case-sensitive (Variable and variable are different).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Make a Python script executable on Unix</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>- Add shebang and set executable permission.
+Example:
+```
+#!/usr/bin/env python3
+# chmod +x script.py
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>self in classes</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>- self refers to the instance inside class methods and accesses attributes.
+Example:
+```
+class User:
+    def __init__(self, name):
+        self.name = name
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Modules vs packages</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>- Module: single .py file.
+- Package: directory of modules with __init__.py.
+Example: import math (module), import numpy.linalg (package).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>PYTHONPATH</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>- Environment variable that tells Python where to look for modules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Global Interpreter Lock (GIL)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>- Only one thread executes Python bytecode at a time.
+- Limits CPU-bound threading; use multiprocessing for parallelism.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Generators</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>- Use yield to produce values lazily and save memory.
+Example:
+```
+def gen():
+    for i in range(3):
+        yield i
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Negative indices</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>- Access elements from the end of a sequence.
+Example: arr[-1] is the last item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>capitalize() and lower()</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>- capitalize() uppercases the first character; lower() makes all lowercase.
+Example:
+```
+'hello'.capitalize()  # 'Hello'
+'Hello'.lower()       # 'hello'
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Ternary operator</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>- Inline conditional expression.
+Example:
+```
+status = 'pass' if score &gt;= 60 else 'fail'
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Dictionary basics</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>- Key-value mapping with unique keys.
+Example:
+```
+user = {'id': 1, 'name': 'Ava'}
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Types of inheritance</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>- Single, multiple, multilevel, and hierarchical inheritance are supported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Polymorphism</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>- Same interface, different implementations.
+- Child classes can override parent methods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Encapsulation</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>- Bundle data and methods; use _ or __ to indicate protected/private.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Abstraction</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>- Expose essential behavior while hiding implementation details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Create an empty class</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>- Use pass to define a class with no members.
+Example:
+```
+class Empty:
+    pass
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>object() usage</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>- object() creates a minimal base object; all classes inherit from object.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Python 2 vs Python 3 differences</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>- Python 3 uses Unicode strings by default and print() is a function.
+- range() returns an iterator-like object (not a list).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Unicode strings in Python 3</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>- str is Unicode; encode/decode to bytes when needed.
+Example:
+```
+text = 'cafe'
+b = text.encode('utf-8')
+```</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Reading files (CSV, Excel, NA values)</t>
         </is>
       </c>
@@ -2703,6 +3379,183 @@
 Example:
 ```
 df_copy = df.copy(deep=True)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Create DataFrame or Series</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>- Construct data structures from lists, dicts, or arrays.
+Example:
+```
+import pandas as pd
+df = pd.DataFrame({'name': ['A', 'B'], 'age': [28, 31]})
+ser = pd.Series([1, 2, 3])
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>query() and filter()</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>- Query with expressions and filter columns by name/pattern.
+Example:
+```
+df.query('age &gt; 30')
+df.filter(['name', 'age'])
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>drop(), rename(), set_index(), reset_index()</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>- Manage columns and indexes.
+Example:
+```
+df = df.drop(columns=['tmp'])
+df = df.rename(columns={'age': 'age_years'})
+df = df.set_index('id')
+df = df.reset_index()
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>pivot_table() and crosstab()</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>- Summarize data in matrix form.
+Example:
+```
+pd.pivot_table(df, index='dept', values='salary', aggfunc='mean')
+pd.crosstab(df['dept'], df['level'])
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>transform() and applymap()</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>- transform returns aligned output; applymap applies elementwise functions.
+Example:
+```
+df.groupby('dept')['salary'].transform('mean')
+df.applymap(lambda x: x*2 if isinstance(x, int) else x)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Resample and shift (time series)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>- Resample by time and shift periods.
+Example:
+```
+df = df.set_index('dt')
+monthly = df.resample('M').sum()
+df['prev'] = df['value'].shift(1)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Visualization: plot, hist, boxplot</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>- Quick charts with built-in plotting.
+Example:
+```
+df.plot(kind='line')
+df['age'].hist()
+df.boxplot(column='salary')
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Write to CSV/Excel</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>- Persist dataframes to files.
+Example:
+```
+df.to_csv('out.csv', index=False)
+df.to_excel('out.xlsx', index=False)
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Statistical functions</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>- Common stats helpers.
+Example:
+```
+df.mean()
+df.median()
+df.std()
+df.min()
+df.max()
+```</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>astype() for type conversion</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>- Convert columns to target dtypes.
+Example:
+```
+df['age'] = df['age'].astype('int64')
 ```</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add playbook sections and spark/cloud details
Co-authored-by: impalalogis <impalalogis@gmail.com>
</commit_message>
<xml_diff>
--- a/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
+++ b/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
@@ -13,6 +13,20 @@
     <sheet name="Section D - Pandas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Section E - PySpark" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Section F - Cloud" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Section 0 - Intro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Section G - CI_CD" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Section I - Lead Scenarios" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Section J - Databricks" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Section K - Migration" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Section L - System Design" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Section M - SQL Practice" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Section N - PySpark Practice" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Section O - Databricks Jobs" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Section P - Behavioral" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Section Q - Arch Visuals" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Section R - Mock QA" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Section H - Spark Optimization" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Section S - Cloud Map" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1611,6 +1625,3124 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Auto Loader</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Delta Lake</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Medallion architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jobs &amp; Workflows</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cluster types</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Unity Catalog basics</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Databricks SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Photon engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Delta Live Tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MLflow basics</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Repos &amp; versioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Secrets management</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Map CDP components to Azure equivalents</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Migrate Hive → Delta</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Migrate Sqoop → ADF/Databricks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Migrate Oozie → ADF/Airflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Migrate HDFS → ADLS Gen2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Security &amp; governance mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Performance tuning differences</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Common migration pitfalls</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Testing &amp; validation strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cutover planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rollback planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> On‑Prem to Databricks Migration Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>“My migration approach follows a structured plan:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Assess current pipelines,</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Identify dependencies,</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Migrate storage to ADLS,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Convert Hive tables to Delta,</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Rewrite Spark jobs in PySpark/SQL,</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Replace Oozie with ADF/Workflows,</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Validate with parallel runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>This ensures minimal downtime and high accuracy.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2. Hive → Delta Conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>“I convert Hive tables to Delta using CTAS or . Delta provides ACID guarantees, schema evolution, and better performance. I also optimize tables with Z‑ORDER and VACUUM.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Code:</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CONVERT TO DELTA hive_metastore.sales USING parquet;</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>3. Sqoop → Auto Loader / ADF</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>“Sqoop is replaced by ADF Copy Activity or Databricks Auto Loader. Auto Loader is ideal for incremental ingestion, while ADF is better for RDBMS extraction.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>4. Oozie → ADF / Databricks Workflows</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>“Oozie workflows map naturally to ADF pipelines or Databricks Workflows. I convert shell actions to notebooks, Hive actions to SQL tasks, and coordinators to triggers.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>5. HDFS → ADLS Migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>“I migrate HDFS data using DistCp or ADF. Folder structure is preserved, and I apply ACLs using Azure AD. After migration, I validate row counts, checksums, and schema.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>6. Parallel Run Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>“I run both old and new pipelines in parallel for 2–4 cycles. I compare aggregates, row counts, and sample records. Any mismatches are fixed before cutover.”</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Batch architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Streaming architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lambda vs Kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lakehouse architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Event-driven pipelines</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Data quality layers</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Metadata &amp; lineage</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>High availability &amp; failover</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Orchestration patterns</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Data modeling best practices</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1. Design a Real‑Time Streaming Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>“I design streaming pipelines using Spark Structured Streaming + Auto Loader + Delta. Data flows from event source → ingestion → bronze → silver → gold. I ensure idempotency, checkpointing, watermarking, and schema evolution. For serving, I use Delta tables or push to downstream systems like Synapse or Power BI.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Key Components:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• </t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Kafka / Event Hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• </t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Auto Loader</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• </t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Delta Bronze/Silver/Gold</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• </t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Checkpointing</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• </t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Watermarking</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• </t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Workflows for orchestration</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2. Design a Data Lakehouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>“A Lakehouse combines data lake storage with warehouse‑style governance. I use ADLS + Delta + Unity Catalog. The architecture follows Bronze → Silver → Gold layers. I enforce schema, optimize tables, and use Z‑ORDER for performance. BI tools connect directly to Gold tables.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>3. Design a Scalable ETL Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>“I build metadata‑driven ETL frameworks where configs define source, target, transformations, and partitioning. The engine reads configs and executes transformations dynamically. This reduces code duplication and improves maintainability.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>4. Design a CDC Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>“I use Delta MERGE for SCD‑1 and SCD‑2. For RDBMS sources, I use ADF incremental extraction or Debezium. I maintain change tables, apply deduplication, and ensure late‑arriving data is handled.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>5. Design a Data Quality Framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>“I define rules like null checks, range checks, referential integrity, and duplicates. I store rules in metadata tables and apply them using PySpark. Failed records go to quarantine tables with error codes.”</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Q_No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Answer_Concept</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Answer_SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Q_No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Answer_Concept</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Answer_Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Brief_Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Job types</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Job clusters vs all-purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Task orchestration</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Parameters &amp; widgets</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ADF/Airflow integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Environments</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alerting &amp; monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Retry &amp; timeout strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Secrets in jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Deployment via CI/CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rollback of jobs</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Sample_Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tell me about yourself</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Biggest project you led</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A time you handled production incident</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Conflict with stakeholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mentoring juniors</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Handling tight deadlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Weakness question</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Why this role/company</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Failure you learned from</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Leadership style</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1. Tell me about a time you handled a production outage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Situation: A critical pipeline failed during month‑end processing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Task: Restore service quickly and prevent data loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Action: I isolated the failing job, checked logs, identified a corrupted input file, applied a hotfix, and re‑ran the pipeline with backfill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Result: Restored service within SLA, prevented revenue impact, and implemented validation checks to avoid recurrence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2. Describe a conflict with a stakeholder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Situation: Product wanted a feature delivered in 2 days; engineering estimated 1 week.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Task: Align expectations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Action: I broke the work into phases, delivered a minimal version in 2 days, and scheduled the rest for the next sprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Result: Stakeholder was satisfied, and the team avoided burnout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>3. Tell me about a time you improved a process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Situation: Manual data validation was taking 3 hours daily.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Task: Automate it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Action: I built a PySpark‑based validation framework with rule‑driven checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Result: Validation time reduced from 3 hours to 10 minutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>4. How do you mentor junior engineers?</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>“I focus on pairing, code reviews, and structured learning paths. I give them ownership of small modules, encourage questions, and help them understand design principles. My goal is to build confidence and autonomy.”</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Diagram_Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ASCII_View</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lakehouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Batch Ingestion</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Streaming</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CI/CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                ┌──────────────────────────────┐</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                │        RAW DATA SOURCES       │</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                │  (RDBMS, APIs, Files, Kafka)  │</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                └───────────────┬──────────────┘</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                │</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                ▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   ┌──────────────────────────┐</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │        BRONZE LAYER       │</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │  Raw, unvalidated data    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │  Auto Loader / Ingestion  │</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   └──────────────┬───────────┘</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                  │</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                  ▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   ┌──────────────────────────┐</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │        SILVER LAYER       │</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │  Cleaned, validated data  │</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │  DQ checks, joins, merges │</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   └──────────────┬───────────┘</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                  │</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                  ▼</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   ┌──────────────────────────┐</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │        GOLD LAYER         │</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │  Aggregates, KPIs, marts  │</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   │  BI-ready tables          │</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                   └──────────────────────────┘</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Q_No</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Suggested_Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Databricks</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Spark</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Spark</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Spark</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DQ</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Behavioral</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1. What is the difference between RDD, DataFrame, and Dataset?</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>“RDD is low‑level and untyped, DataFrame is optimized and schema‑based, Dataset is typed but available only in Scala/Java. In practice, I use DataFrames because they leverage Catalyst and Tungsten optimizations.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2. How do you handle skew in Spark?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>“I detect skew using Spark UI, then fix it using salting, broadcast joins, or repartitioning. For extreme skew, I apply range partitioning or pre‑aggregation.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>3. What is Z‑ORDER in Delta?</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>“Z‑ORDER optimizes data skipping by co‑locating related values. It improves performance for selective queries.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>4. How do you design a CDC pipeline?</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>“I ingest incremental data, dedupe using window functions, and apply MERGE INTO for SCD‑1 or SCD‑2. I maintain audit columns and handle late‑arriving data.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>5. How do you ensure data quality?</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Answer:</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>“I define rules (null checks, referential integrity, duplicates), store them in metadata tables, and apply them using PySpark. Failed records go to quarantine tables.”</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C79"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Driver, Executors, Cluster Manager</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Driver schedules work, executors run tasks, cluster manager allocates resources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RDD vs DataFrame vs Dataset</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RDD is low-level; DataFrame is optimized; Dataset adds types in Scala.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Lazy evaluation</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Builds a DAG; execution starts only when an action runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Transformations vs Actions</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Transformations create lineage; actions trigger execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Narrow vs Wide transformations</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Narrow does not shuffle; wide triggers shuffle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Catalyst Optimizer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Optimizes logical and physical plans for DataFrame and SQL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tungsten engine</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Uses binary processing and codegen for CPU efficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Shuffle mechanics</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Shuffle moves data across partitions and is expensive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Broadcast variables</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Broadcast small reference data to executors for fast lookups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Accumulators</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Write-only shared variables for metrics and counters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Caching &amp; persistence</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Cache only reused dataframes; unpersist after use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Partitioning &amp; coalescing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Partition by high-cardinality columns for parallelism; low-cardinality for pruning. Use coalesce to reduce partitions without shuffle; repartition for balancing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Adaptive Query Execution (AQE)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Enable AQE to auto-optimize joins, skew, and partitions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Delta Lake internals</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Transaction log enables ACID, schema enforcement, and time travel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Broadcast join optimization</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Use broadcast for small lookup tables to avoid shuffle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Avoid wide shuffles</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Minimize shuffles by filtering early and pre-aggregating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Repartition vs Coalesce</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Use coalesce to reduce partitions without shuffle; repartition for balancing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Avoid UDFs</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Use built-in functions or Pandas UDFs for vectorization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>File size optimization</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Target 128-512 MB file sizes to avoid small file problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Use explain()</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Inspect query plans to find expensive stages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Handling skew</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Add random salt to distribute skewed keys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Checkpointing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Break lineage to avoid stack overflow and memory issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Z-Ordering</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Improve data skipping for selective queries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>OPTIMIZE + VACUUM</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Compact small files and improve read performance. Remove obsolete files to reduce storage and metadata overhead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Auto Loader best practices</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Efficient file discovery and schema evolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Spark Concepts</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Cluster sizing &amp; autoscaling</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Right-size executors and scale workers based on workload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Partitioning Strategy</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Partition by high-cardinality columns for parallelism; low-cardinality for pruning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Broadcast Joins</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Use broadcast for small lookup tables to avoid shuffle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Caching &amp; Persisting</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Cache only reused dataframes; unpersist after use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Avoid Wide Transformations</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Minimize shuffles by filtering early and pre-aggregating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Coalesce vs Repartition</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Use coalesce to reduce partitions without shuffle; repartition for balancing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Z-ORDER Clustering</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Improve data skipping for selective queries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>File Size Tuning</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Target 128-512 MB file sizes to avoid small file problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Predicate Pushdown</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Push filters to the data source to reduce scan volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Column Pruning</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Select only required columns to reduce memory usage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Avoid Python UDFs</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Use built-in functions or Pandas UDFs for vectorization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Broadcast Hint</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Force broadcast when Spark does not auto-broadcast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Skew Handling with Salting</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Add random salt to distribute skewed keys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Optimize Shuffle Partitions</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Tune spark.sql.shuffle.partitions based on cluster size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Use Delta Lake OPTIMIZE</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Compact small files and improve read performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Use Checkpointing for Long Lineages</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Break lineage to avoid stack overflow and memory issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Avoid Collect()</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Never bring large datasets to the driver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Use mapPartitions Instead of map</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Process data in batches for performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Avoid Explode on Large Arrays</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Explode causes massive shuffles; pre-filter arrays first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Use Bloom Filters</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Enable bloom filters for faster joins on Delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Use Data Skipping Statistics</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Delta stores min/max stats for skipping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Use Photon Engine (Databricks)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Photon accelerates SQL and Delta workloads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Use Auto Loader for Incremental Ingestion</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Efficient file discovery and schema evolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Use Delta MERGE Instead of Manual Upserts</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Optimized for CDC and SCD-2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Use VACUUM to Clean Old Files</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Remove obsolete files to reduce storage and metadata overhead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Use OPTIMIZE WRITE</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Databricks feature to auto-compact files during write.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Use Liquid Clustering (Databricks)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Next-gen clustering for large Delta tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Avoid Cross Joins</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Unless absolutely necessary; they explode data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Use Window Functions Carefully</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Window functions cause shuffles; partition wisely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Use Range Partitioning for Time-Series</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Partition by date for pruning and parallelism.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Use Incremental ETL Instead of Full Loads</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Reduces compute cost and improves latency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Use Bloom Filter Indexes</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Accelerate point-lookups on Delta tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Use Delta Change Data Feed (CDF)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Efficient incremental processing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Use Auto-Optimize (Databricks)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Automatically compacts small files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Optimization Tips</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Avoid Repeated Reads</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Cache or checkpoint instead of re-reading from storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Spark Optimization Cheatsheet</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Shuffles</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Avoid wide transformations, use broadcast joins, reduce shuffle partitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Spark Optimization Cheatsheet</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Skew</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Salting, AQE skew join optimization, range partitioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Spark Optimization Cheatsheet</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Use Delta, OPTIMIZE, Z-ORDER, compact files</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Spark Optimization Cheatsheet</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Avoid collect(), prune columns, use mapPartitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Spark Optimization Cheatsheet</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Tune partitions, autoscaling, Photon engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Spark Optimization Cheatsheet</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ETL</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Incremental loads, MERGE INTO, Auto Loader</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Spark Optimization Cheatsheet</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Use Unity Catalog, enforce schema, use CDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Databricks Tuning</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>DBR Versions</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Use DBR 13+ for best performance. DBR 14.x supports Photon 3.0, Liquid Clustering, improved AQE, better Delta performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Databricks Tuning</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Photon Engine</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Vectorized C++ engine; 2-5x faster SQL. Enable via Photon clusters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Databricks Tuning</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Autoscaling</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Min workers for baseline, max for peak load. Use optimized autoscaling for faster ramp-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Databricks Tuning</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Auto-Optimize</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Automatically compacts files and optimizes writes. Enable at cluster or table level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Databricks Tuning</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Liquid Clustering</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Next-gen clustering for large Delta tables with Z-ORDER-like skipping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Cluster Sizing</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Executor Sizing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>4-8 cores per executor, 16-32 GB RAM per executor; avoid too many small executors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Cluster Sizing</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Driver Sizing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Driver = 1.5x executor memory; limit collect() to avoid OOM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Cluster Sizing</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Partition Sizing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>128-512 MB per partition; num_partitions = total_data_size / 256MB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Cluster Sizing</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Worker Node Count</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Heavy ETL: 8-16 nodes; Streaming: 2-4 nodes; ML: GPU nodes if needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Cluster Sizing</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Autoscaling Strategy</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Min workers = 2, Max workers = 10-20; use optimized autoscaling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Cluster Sizing</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SQL Warehouse Sizing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Use Pro for BI, Serverless for ad-hoc queries; scale by concurrency.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1855,6 +4987,425 @@
 - Design for data quality and consistent definitions.
 - Balance normalization vs performance.
 - Plan for scalability and document the model.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Service Category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CDP</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Azure</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>GCP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CI/CD</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bitbucket, Jenkins, RLM DevOps</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Azure DevOps, GitHub Enterprise</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AWS CodeBuild, CodeDeploy, CodePipeline</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cloud Build, Cloud Deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Data Warehouse</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hive, Impala</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Azure Synapse Analytics</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Amazon Redshift</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BigQuery</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Data Integration</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PySpark + Shell, NiFi, Sqoop</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Azure Data Factory</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AWS Glue, Amazon Data Pipeline</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cloud Data Fusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Messaging</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JMS, Kafka</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Azure Service Bus, Event Hubs</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Amazon Kinesis, SNS, SQS</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Google Pub/Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Workflow Orchestration</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Oozie, Autosys, Airflow</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Azure Data Factory, Azure Logic Apps</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AWS Step Functions, Glue Workflows, Airflow</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Cloud Composer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Document DB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>N/A or HBase</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Azure Cosmos DB</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Amazon DocumentDB</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Firestore</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NoSQL (Key/Value)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HBase</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Azure Cosmos DB</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Amazon DynamoDB</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Cloud Bigtable</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RDBMS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Hive, Impala, Oracle (external)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Azure SQL Database</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Amazon Aurora, Amazon RDS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Cloud SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Storage Transfer</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DistCp, NiFi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Azure Data Factory, Storage Mover</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AWS Storage Gateway, DataSync</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Storage Transfer Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Network Connectivity</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Knox Gateway, SDX</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Azure VPN Gateway</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>AWS VPN</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Cloud VPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Audit Logging</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ranger Audit, Cloudera Navigator</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Azure Monitor, Azure Audit Logs</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>AWS CloudTrail</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Cloud Audit Logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Key Management</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CyberArk, Ranger KMS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Azure Key Vault</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>AWS KMS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Cloud KMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Identity Management</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>LDAP, Sentry, Ranger</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Azure Active Directory</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>AWS IAM</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Google Cloud IAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HDFS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Azure Blob Storage (ADLS Gen2)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Amazon S3</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Google Cloud Storage</t>
         </is>
       </c>
     </row>
@@ -3929,4 +7480,617 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Profile Summary</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>13+ years Data Engineering experience across Cloudera, Azure Databricks, ETL, Data Quality, Governance</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Core Skills</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Python, SQL, Shell Scripting, Data Modeling, Data Quality, Agile Scrum</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cloud Platforms</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cloudera CDP/CDH, Azure, AWS, GCP, Databricks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ETL Tools</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Azure Data Factory, Databricks, SSIS, Informatica</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Big Data Technologies</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Spark, PySpark, Hadoop, HDFS, Hive, Pig, Sqoop, Kafka</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CI/CD &amp; Automation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Jenkins, RLM DevOps, Git, GitHub, Bitbucket</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Migration Experience</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Migration from Cloudera pipelines to Azure Databricks Lakehouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>REST API Integration</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Python REST API development for data ingestion and conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>🟦 INTRO SHEET — FULL A2‑LEVEL CONTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Below are the rows you should add to the Intro sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1. Profile Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Details:</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>“I’m a Senior/Lead Data Engineer with deep experience across Databricks, Spark, PySpark, SQL, and cloud data platforms. My work spans end‑to‑end data engineering — ingestion, transformation, modeling, optimization, and production operations. I’ve led migrations from on‑prem Hadoop/Cloudera to Azure Databricks, built Lakehouse architectures, and designed scalable ETL frameworks. My focus is on reliability, performance, governance, and building systems that scale with business growth.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2. Technical Strengths</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Details:</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>“My core strengths include distributed data processing (Spark/PySpark), SQL optimization, Delta Lake, Databricks Workflows, ADF, and metadata‑driven ETL frameworks. I’m strong in Python automation, CI/CD, and designing modular, reusable pipelines. I also bring experience in data modeling, CDC, streaming, and data quality engineering.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3. Cloud &amp; Platform Expertise</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Details:</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>“I’ve worked extensively on Azure (ADLS, ADF, Databricks, Key Vault), AWS (S3, Glue, EMR), and Cloudera (CDH/CDP). My strongest area is Azure Databricks, where I build Lakehouse architectures using Delta, Auto Loader, and Unity Catalog. I design pipelines that are secure, cost‑efficient, and easy to operate.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>4. End‑to‑End ETL/ELT Experience</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Details:</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>“I design ETL/ELT pipelines following Bronze → Silver → Gold architecture. My pipelines are modular, parameterized, and metadata‑driven. I implement incremental loads, schema evolution, and CDC using Delta MERGE. I also build monitoring, alerting, and audit frameworks to ensure reliability.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>5. Leadership &amp; Ownership</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Details:</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>“I’ve led teams of data engineers, driven architectural decisions, and owned critical production pipelines. I focus on clarity, accountability, and building a culture of high‑quality engineering. I mentor junior engineers, run code reviews, and ensure best practices across the team.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>6. Migration Experience</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Details:</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>“I’ve led large‑scale migrations from Cloudera/Hadoop to Azure Databricks. This includes data transfer, Hive‑to‑Delta conversion, Spark job rewriting, Oozie‑to‑ADF migration, and parallel run validation. I ensure schema alignment, performance tuning, and governance compliance during migration.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>7. Data Quality &amp; Governance</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Details:</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>“I design rule‑driven data quality frameworks with null checks, referential integrity, duplicates, and anomaly detection. I use Unity Catalog for governance, lineage, and access control. I ensure pipelines are audit‑ready and compliant with organizational standards.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>8. Business Impact</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Details:</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>“My work has improved pipeline performance, reduced operational overhead, and enabled faster analytics. I’ve automated manual processes, reduced processing time by 40–70%, and built systems that support real‑time and batch workloads. I focus on delivering measurable business value.”</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Git clone, pull, push, fetch</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Git branching strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Git merge vs rebase</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Git stash</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Git revert vs reset</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jenkins pipeline stages</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Build → Test → Deploy flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CI triggers (webhooks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CD deployment strategies</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rollback strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Versioning &amp; tagging</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Code review best practices</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Brief_Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Design end-to-end Databricks + ADF pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Design Lakehouse architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Migrate Cloudera to Azure Databricks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Handle schema evolution in Delta Lake</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Design CDC ingestion</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Build Medallion architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Reduce 3-hour Spark job</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Handle data skew</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Optimize SQL queries</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Reduce shuffle operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Optimize ADF pipelines</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Implement DQ checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Enforce schema validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Design audit logging</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Handle PII data</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CI/CD for Databricks notebooks</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Version control strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Deployment automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rollback strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Debug failing Spark jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Recover corrupted Delta tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Handle accidental deletes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Manage 2 AM pipeline failures</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Mentor junior engineers</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Handle conflicting requirements</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Communicate delays</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ensure cross-team alignment</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refine Python and Pandas interview sections
Co-authored-by: impalalogis <impalalogis@gmail.com>
</commit_message>
<xml_diff>
--- a/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
+++ b/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
@@ -5420,7 +5420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5440,1203 +5440,638 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Shallow copy vs deep copy</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>- Shallow copy copies the outer container; nested objects are shared.
-- Deep copy recursively copies nested objects.
-Example:
-```
-import copy
-x = [[1, 2], [3, 4]]
-sh = copy.copy(x)
-dp = copy.deepcopy(x)
-sh[0].append(99)
-# x changes, dp does not
-```</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Python characteristics</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Interpreted and dynamically typed; types checked at runtime.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Multithreading in Python</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>- Use threading for IO-bound tasks; GIL limits CPU-bound parallelism.
-Example:
-```
-from threading import Thread
-def fetch(url):
-    ...
-threads = [Thread(target=fetch, args=(u,)) for u in urls]
-[t.start() for t in threads]
-[t.join() for t in threads]
-```</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Python case sensitivity</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Identifiers are case-sensitive.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Django architecture</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>- Django follows MTV: Model (ORM), Template (UI), View (request logic).
-- URL dispatcher and middleware connect requests to views.
-Example:
-```
-# urls.py
-path('users/', views.user_list)
-# views.py
-return render(request, 'users.html', {'users': User.objects.all()})
-```</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PEP 8</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Style guide for readable, consistent Python.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Keywords in Python</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reserved words; cannot be used as identifiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Python namespaces (LEGB)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Name resolution order: Local, Enclosing, Global, Builtins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Global vs local variables</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Local inside function; global at module scope; use global to rebind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>__name__ and main guard</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>When run directly, __name__ == '__main__'; use guard for entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pass-by-object reference</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Arguments pass references; mutation affects caller, rebinding does not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>List vs tuple</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>List is mutable; tuple is immutable and can be hashable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dictionary basics</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Key-value mapping with unique keys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Merge elements in sequences</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Use + for concat, itertools.chain for iterables, zip for pairing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>append() vs extend()</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>append adds one object; extend adds elements from an iterable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>del vs remove()</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>del removes by index/name; remove deletes first matching value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Slicing</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>seq[start:stop:step], stop is exclusive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Negative indices</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Index from end; -1 is last element.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Common string ops</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>split/replace/strip/isalnum/lower/capitalize are common string helpers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>// operator</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Floor division; rounds down for positives and negatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>is vs ==</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>is checks identity; == checks value equality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ternary operator</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>expr_if_true if condition else expr_if_false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>continue vs break vs pass</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>continue skips iteration; break exits loop; pass is no-op.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Docstrings</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>First string literal documents object; available via __doc__.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>First-class functions</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Functions can be assigned, passed, and returned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>*args and **kwargs</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Collect variable positional and keyword arguments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Lambda functions</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Anonymous single-expression functions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Decorators</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Wrap functions to add behavior without changing body.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Iterators</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Implement __iter__/__next__; use iter() and next().</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Generators</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Use yield for lazy sequences and lower memory use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Random number generation</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Use random for general RNG; secrets for crypto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Pickling vs unpickling</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>- Pickling serializes objects to bytes; unpickling restores them.
-Example:
-```
-import pickle
-blob = pickle.dumps({'a': 1})
-obj = pickle.loads(blob)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Memory management in Python</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>- Uses reference counting plus cyclic GC; small objects use pymalloc arenas.
-Example:
-```
-import gc
-obj = []
-obj.append(obj)
-del obj
-gc.collect()
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Pass-by-reference vs pass-by-value</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>- Python passes object references (call-by-object).
-- Mutating a passed mutable affects the caller; rebinding does not.
-Example:
-```
-def f(lst):
-    lst.append(1)
-a = []
-f(a)  # a becomes [1]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Random number generation</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>- Use random for general RNG, seed for reproducibility; use secrets for crypto.
-Example:
-```
-import random
-random.seed(42)
-random.randint(1, 10)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>// operator</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>- Floor division; result is the floor of true division.
-Example:
-```
-7 // 3   # 2
--7 // 3  # -3
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>"is" operator</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>- Checks object identity, not equality.
-Example:
-```
-a = [1]
-b = [1]
-(a == b)  # True
-(a is b)  # False
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>pass statement</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>- No-op placeholder used where syntax requires a statement.
-Example:
-```
-def todo():
-    pass
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Check if string is alphanumeric</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>- Use str.isalnum().
-Example:
-```
-'sku123'.isalnum()  # True
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Merge elements in sequences</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>- Concatenate or chain sequences; zip to pair elements.
-Example:
-```
-import itertools
-merged = list(itertools.chain([1, 2], [3, 4]))
-paired = list(zip([1, 2], ['a', 'b']))
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Remove leading whitespace</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>- Use lstrip().
-Example:
-```
-'  abc'.lstrip()  # 'abc'
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>replace() usage</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>- Replace substrings with str.replace(old, new, count).
-Example:
-```
-'2026-01-26'.replace('-', '/')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>del vs remove()</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>- del deletes by index or deletes a name; remove deletes first matching value.
-Example:
-```
-a = [1, 2, 3]
-del a[0]    # [2, 3]
-a.remove(3) # [2]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>append() vs extend()</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>- append adds one object; extend adds elements from an iterable.
-Example:
-```
-a = [1]
-a.append([2, 3])  # [1, [2, 3]]
-a.extend([4, 5])  # [1, [2, 3], 4, 5]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Serialize objects to bytes and restore later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Memory management</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Reference counting plus cyclic garbage collection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GIL and multithreading</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>One thread runs bytecode; threading best for IO-bound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Make script executable (Unix)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Add shebang and chmod +x script.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Modules vs packages</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Module is a .py file; package is a directory with __init__.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PYTHONPATH</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Environment variable that adds module search paths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>self in classes</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Instance reference used to access attributes and methods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Inheritance types</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Single, multiple, multilevel, hierarchical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Polymorphism</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Same interface, different implementations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Encapsulation</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bundle data/methods; use _ or __ for non-public.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Abstraction</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Expose essentials while hiding implementation details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Create an empty class</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>class Empty: pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>object() usage</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Minimal base object; all classes inherit from object.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Python 2 vs Python 3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Python 3 has Unicode str, print() function, lazy range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Unicode strings</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>str is Unicode; encode to bytes with utf-8 when needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Django architecture (MTV)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Model = data, Template = UI, View = request logic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Reverse file contents</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>- Read lines and write/print in reverse order.
-Example:
-```
-with open('f.txt') as f:
-    lines = f.readlines()
-rev = ''.join(reversed(lines))
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>List vs Tuple</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>- List is mutable; tuple is immutable and can be hashable.
-Example:
-```
-coords = (10, 20)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Docstring</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>- First string literal in a module/class/function; available via __doc__.
-Example:
-```
-def add(a, b):
-    'Return sum of a and b.'
-    return a + b
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>split() function</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>- str.split(sep, maxsplit) splits a string into a list.
-Example:
-```
-'foo,bar'.split(',')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>*args and **kwargs</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>- *args collects positional args; **kwargs collects keyword args.
-Example:
-```
-def f(*args, **kwargs):
-    return args, kwargs
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>First-class functions</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>- Functions can be assigned, passed, and returned like data.
-Example:
-```
-def apply(f, x):
-    return f(x)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>What is __name__</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>- Module name; when run directly, __name__ == '__main__'.
-Example:
-```
-if __name__ == '__main__':
-    main()
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Read lines and reverse before output or writing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>NumPy arrays</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>- N-dimensional, homogeneous arrays with vectorized operations.
-Example:
-```
-import numpy as np
-arr = np.array([1, 2, 3])
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Homogeneous n-D arrays with vectorized operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Matrices vs arrays</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>- Arrays are general n-D; matrices are strictly 2-D. Prefer arrays with @.
-Example:
-```
-A = np.array([[1, 2], [3, 4]])
-B = np.array([[5, 6], [7, 8]])
-A @ B
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>argsort usage</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>- Returns indices that would sort an array.
-Example:
-```
-import numpy as np
-x = np.array([30, 10, 20])
-idx = np.argsort(x)  # [1, 2, 0]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>vstack usage</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>- Stack arrays vertically (row-wise).
-Example:
-```
-import numpy as np
-np.vstack([[1, 2], [3, 4]])
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Matrix is 2-D; array is n-D; use @ for matmul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>argsort and vstack</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>argsort gives sort indices; vstack stacks arrays row-wise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sort array by column</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Use arr[arr[:, col].argsort()] for column sort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>DecisionTree import</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>- Import from sklearn.tree.
-Example:
-```
-from sklearn.tree import DecisionTreeClassifier
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Pandas read_csv encoding issue</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>- Specify encoding and error handling.
-Example:
-```
-import pandas as pd
-df = pd.read_csv('data.csv', encoding='latin1', errors='replace')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Matplotlib linewidth</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>- Use linewidth (or lw) in plotting calls.
-Example:
-```
-import matplotlib.pyplot as plt
-plt.plot(x, y, linewidth=2)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>reindex vs reset_index</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>- reindex changes index labels/ordering; reset_index moves index to a column.
-Example:
-```
-df = df.reindex(['b', 'a'])
-df = df.reset_index(drop=True)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>xrange vs range</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>- Python2: xrange is lazy, range builds list. Python3: range is lazy; xrange removed.
-Example:
-```
-for i in range(3):
-    print(i)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Check if DataFrame is empty</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>- Use df.empty (True if no rows or columns).
-Example:
-```
-df.empty
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Sort array by column</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>- Use argsort on the target column.
-Example:
-```
-import numpy as np
-arr = np.array([[3, 1], [2, 9], [1, 5]])
-arr[arr[:, 0].argsort()]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Create Series from list/array/dict</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>- Use pd.Series with different inputs.
-Example:
-```
-import pandas as pd
-pd.Series([1, 2])
-pd.Series({'a': 1, 'b': 2})
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Items not common between two Series</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>- Use symmetric difference with isin.
-Example:
-```
-import pandas as pd
-s1 = pd.Series([1, 2, 3])
-s2 = pd.Series([2, 3, 4])
-not_common = pd.concat([s1[~s1.isin(s2)], s2[~s2.isin(s1)]])
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Replace all except top 2 frequent values</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>- Keep top 2 values, replace others.
-Example:
-```
-import pandas as pd
-s = pd.Series(['a', 'b', 'a', 'c', 'd', 'a', 'b'])
-top2 = s.value_counts().nlargest(2).index
-s2 = s.where(s.isin(top2), other='Other')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Find multiples of 3 in Series</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>- Filter using modulo.
-Example:
-```
-import pandas as pd
-s = pd.Series([1, 3, 4, 6])
-mult3 = s[s % 3 == 0]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Euclidean distance between Series</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>- Compute norm of the difference.
-Example:
-```
-import numpy as np
-import pandas as pd
-s1 = pd.Series([1, 2, 3])
-s2 = pd.Series([4, 5, 6])
-dist = np.linalg.norm(s1 - s2)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Reverse DataFrame rows</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>- Reverse with iloc and reset index.
-Example:
-```
-df_rev = df.iloc[::-1].reset_index(drop=True)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Overfitting with train/test split</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>- Overfitting shows strong train but weak test performance.
-- Mitigate with validation, cross-validation, regularization, and simpler models.
-Example:
-```
-from sklearn.model_selection import train_test_split
-X_train, X_test, y_train, y_test = train_test_split(X, y, test_size=0.2, random_state=42)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Seaborn usage</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>- High-level statistical plotting built on matplotlib.
-Example:
-```
-import seaborn as sns
-sns.barplot(data=df, x='dept', y='salary')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Python literals</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>- Fixed values in source code: numbers, strings, bytes, booleans, None, collections.
-Example:
-```
-42, 3.14, 'text', b'bin', True, None, [1, 2], {'a': 1}
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Decorators</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>- Functions that wrap other functions to add behavior.
-Example:
-```
-def log_call(f):
-    def wrapper(*args, **kwargs):
-        print(f.__name__)
-        return f(*args, **kwargs)
-    return wrapper
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Slicing</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>- Use start:stop:step; stop is exclusive.
-Example:
-```
-arr = [0, 1, 2, 3, 4]
-arr[1:4:2]  # [1, 3]
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Keywords in Python</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>- Reserved words that cannot be identifiers; see keyword.kwlist.
-Example:
-```
-import keyword
-keyword.kwlist
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Lambda functions</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>- Anonymous, single-expression functions.
-Example:
-```
-add = lambda x, y: x + y
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>continue vs break vs pass</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>- continue skips to next iteration; break exits loop; pass does nothing.
-Example:
-```
-for i in range(3):
-    if i == 1:
-        continue
-    if i == 2:
-        break
-    pass
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Iterators</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>- Iterators implement __iter__ and __next__; use iter() and next().
-Example:
-```
-it = iter([1, 2, 3])
-next(it)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Python namespaces</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>- Namespaces map names to objects; scope order is LEGB.
-Example:
-```
-x = 1
-def f():
-    x = 2  # local
-```</t>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>from sklearn.tree import DecisionTreeClassifier.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Python features (interpreted, dynamically typed)</t>
+          <t>Matplotlib linewidth</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>- Python is interpreted and dynamically typed; types are checked at runtime.
-- Enables rapid development and flexibility.</t>
+          <t>Use linewidth or lw parameter in plot().</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PEP 8</t>
+          <t>Seaborn usage</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>- Python Enhancement Proposal for style and formatting.
-- Consistent naming, indentation, and readability guidelines.</t>
+          <t>High-level statistical plotting on matplotlib.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Global vs local variables</t>
+          <t>Overfitting with train/test split</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>- Local variables live inside a function.
-- Global variables are defined at module scope and accessible everywhere.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Python case sensitivity</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>- Python is case-sensitive (Variable and variable are different).</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Make a Python script executable on Unix</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>- Add shebang and set executable permission.
-Example:
-```
-#!/usr/bin/env python3
-# chmod +x script.py
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>self in classes</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>- self refers to the instance inside class methods and accesses attributes.
-Example:
-```
-class User:
-    def __init__(self, name):
-        self.name = name
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Modules vs packages</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>- Module: single .py file.
-- Package: directory of modules with __init__.py.
-Example: import math (module), import numpy.linalg (package).</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>PYTHONPATH</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>- Environment variable that tells Python where to look for modules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Global Interpreter Lock (GIL)</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>- Only one thread executes Python bytecode at a time.
-- Limits CPU-bound threading; use multiprocessing for parallelism.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Generators</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>- Use yield to produce values lazily and save memory.
-Example:
-```
-def gen():
-    for i in range(3):
-        yield i
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Negative indices</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>- Access elements from the end of a sequence.
-Example: arr[-1] is the last item.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>capitalize() and lower()</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>- capitalize() uppercases the first character; lower() makes all lowercase.
-Example:
-```
-'hello'.capitalize()  # 'Hello'
-'Hello'.lower()       # 'hello'
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Ternary operator</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>- Inline conditional expression.
-Example:
-```
-status = 'pass' if score &gt;= 60 else 'fail'
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Dictionary basics</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>- Key-value mapping with unique keys.
-Example:
-```
-user = {'id': 1, 'name': 'Ava'}
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Types of inheritance</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>- Single, multiple, multilevel, and hierarchical inheritance are supported.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Polymorphism</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>- Same interface, different implementations.
-- Child classes can override parent methods.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Encapsulation</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>- Bundle data and methods; use _ or __ to indicate protected/private.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Abstraction</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>- Expose essential behavior while hiding implementation details.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Create an empty class</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>- Use pass to define a class with no members.
-Example:
-```
-class Empty:
-    pass
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>object() usage</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>- object() creates a minimal base object; all classes inherit from object.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Python 2 vs Python 3 differences</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>- Python 3 uses Unicode strings by default and print() is a function.
-- range() returns an iterator-like object (not a list).</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Unicode strings in Python 3</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>- str is Unicode; encode/decode to bytes when needed.
-Example:
-```
-text = 'cafe'
-b = text.encode('utf-8')
-```</t>
+          <t>High train, low test; mitigate with validation/regularization.</t>
         </is>
       </c>
     </row>
@@ -6671,443 +6106,302 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Reading files (CSV, Excel, NA values)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>- Use pandas readers and control NA parsing.
-Example:
-```
-import pandas as pd
-df = pd.read_csv('data.csv', na_values=['NA', ''], keep_default_na=True)
-xl = pd.read_excel('data.xlsx', sheet_name='Sheet1')
-```</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Create DataFrame/Series</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Use pd.DataFrame or pd.Series from list, dict, or array.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Data exploration (head, info, describe)</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>- Inspect shape and summary statistics.
-Example:
-```
-df.head()
-df.info()
-df.describe()
-```</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Read/Write CSV/Excel</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>read_csv/read_excel; to_csv/to_excel; set encoding if needed.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Data types &amp; conversions</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>- Check dtypes and convert using astype/to_numeric/to_datetime.
-Example:
-```
-df.dtypes
-df['age'] = df['age'].astype('int')
-df['dt'] = pd.to_datetime(df['dt'])
-```</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Data exploration</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>head, tail, info, describe, shape for quick profiling.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Indexing: loc, iloc, at, iat</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>- loc/at are label-based; iloc/iat are position-based.
-Example:
-```
-df.loc[5, 'name']
-df.iloc[5, 0]
-df.at[5, 'name']
-df.iat[5, 0]
-```</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Data types &amp; conversion</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>dtypes, astype, to_numeric, to_datetime.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Filtering, conditions, isin, between</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>- Build boolean masks and filter.
-Example:
-```
-df[df['salary'] &gt; 100000]
-df[df['dept'].isin(['IT', 'HR'])]
-df[df['age'].between(25, 40)]
-```</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Indexing: loc/iloc/at/iat</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>loc/at label-based; iloc/iat position-based.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Aggregations, groupby, agg</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>- Group by keys and compute aggregates.
-Example:
-```
-df.groupby('dept').agg({'salary': 'mean', 'emp_id': 'count'})
-```</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Filtering</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Boolean masks, query(), isin(), between().</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Removing duplicates (rows &amp; columns)</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>- Drop duplicate rows or duplicate columns.
-Example:
-```
-df = df.drop_duplicates()
-df = df.loc[:, ~df.columns.duplicated()]
-```</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Missing values</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>isnull/notnull, fillna, dropna.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Missing values: isnull, fillna, dropna</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>- Detect and handle nulls.
-Example:
-```
-df.isnull().sum()
-df['city'] = df['city'].fillna('Unknown')
-df = df.dropna(subset=['salary'])
-```</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Duplicates</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>duplicated and drop_duplicates; columns via df.columns.duplicated.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Sorting, nlargest, nsmallest</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>- Sort rows or take top/bottom N.
-Example:
-```
-df.sort_values('salary', ascending=False)
-df.nlargest(5, 'salary')
-df.nsmallest(5, 'salary')
-```</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sorting</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sort_values/sort_index; nlargest/nsmallest for top/bottom.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>concat, merge, join</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>- Combine DataFrames by rows, columns, or keys.
-Example:
-```
-pd.concat([df1, df2], axis=0)
-df1.merge(df2, on='id', how='left')
-df1.join(df2.set_index('id'), on='id')
-```</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Reindex vs reset_index</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>reindex aligns labels; reset_index moves index to column.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Groupby/agg/transform</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>groupby keys, agg metrics; transform returns aligned output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Merge/join/concat</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>merge on keys, join on index, concat rows or columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pivot/crosstab</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>pivot_table for aggregates; crosstab for counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>String operations</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>- Use vectorized string methods.
-Example:
-```
-df['name'].str.lower()
-df['email'].str.contains('@')
-df['city'].str.replace(' ', '_')
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Use Series.str methods like lower, contains, replace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Datetime operations</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>- Parse dates and use dt accessor or resample.
-Example:
-```
-df['dt'] = pd.to_datetime(df['dt'])
-df['year'] = df['dt'].dt.year
-monthly = df.set_index('dt').resample('M').sum()
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Apply, map, vectorize</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>- Prefer vectorized ops; apply/map for custom logic.
-Example:
-```
-df['score2'] = df['score'].map(lambda x: x * 2)
-df['flag'] = df.apply(lambda r: r['a'] &gt; r['b'], axis=1)
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Clipping, replacing values</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>- Clip outliers and replace values.
-Example:
-```
-df['pct'] = df['pct'].clip(lower=0, upper=100)
-df['status'] = df['status'].replace({'Y': 'Yes', 'N': 'No'})
-```</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Copying DataFrames</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>- Use copy to avoid chained assignment issues.
-Example:
-```
-df_copy = df.copy(deep=True)
-```</t>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>to_datetime, dt accessor, resample, shift.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Create DataFrame or Series</t>
+          <t>Apply/map/vectorize</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>- Construct data structures from lists, dicts, or arrays.
-Example:
-```
-import pandas as pd
-df = pd.DataFrame({'name': ['A', 'B'], 'age': [28, 31]})
-ser = pd.Series([1, 2, 3])
-```</t>
+          <t>map for Series; apply for rows/cols; applymap elementwise.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>query() and filter()</t>
+          <t>Replace/clip</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>- Query with expressions and filter columns by name/pattern.
-Example:
-```
-df.query('age &gt; 30')
-df.filter(['name', 'age'])
-```</t>
+          <t>replace values; clip bounds outliers.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>drop(), rename(), set_index(), reset_index()</t>
+          <t>Copying DataFrames</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>- Manage columns and indexes.
-Example:
-```
-df = df.drop(columns=['tmp'])
-df = df.rename(columns={'age': 'age_years'})
-df = df.set_index('id')
-df = df.reset_index()
-```</t>
+          <t>Use df.copy() to avoid chained assignment side effects.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>pivot_table() and crosstab()</t>
+          <t>Check if DataFrame is empty</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>- Summarize data in matrix form.
-Example:
-```
-pd.pivot_table(df, index='dept', values='salary', aggfunc='mean')
-pd.crosstab(df['dept'], df['level'])
-```</t>
+          <t>df.empty is True when no rows or columns.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>transform() and applymap()</t>
+          <t>Reverse DataFrame rows</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>- transform returns aligned output; applymap applies elementwise functions.
-Example:
-```
-df.groupby('dept')['salary'].transform('mean')
-df.applymap(lambda x: x*2 if isinstance(x, int) else x)
-```</t>
+          <t>df.iloc[::-1].reset_index(drop=True).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Resample and shift (time series)</t>
+          <t>Series difference</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>- Resample by time and shift periods.
-Example:
-```
-df = df.set_index('dt')
-monthly = df.resample('M').sum()
-df['prev'] = df['value'].shift(1)
-```</t>
+          <t>Use isin to keep values not present in the other Series.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Visualization: plot, hist, boxplot</t>
+          <t>Top-N frequency replace</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>- Quick charts with built-in plotting.
-Example:
-```
-df.plot(kind='line')
-df['age'].hist()
-df.boxplot(column='salary')
-```</t>
+          <t>Use value_counts().nlargest(N) to keep top values.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Write to CSV/Excel</t>
+          <t>Series modulo filtering</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>- Persist dataframes to files.
-Example:
-```
-df.to_csv('out.csv', index=False)
-df.to_excel('out.xlsx', index=False)
-```</t>
+          <t>Filter with s[s % k == 0] for divisibility.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Statistical functions</t>
+          <t>Euclidean distance between Series</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>- Common stats helpers.
-Example:
-```
-df.mean()
-df.median()
-df.std()
-df.min()
-df.max()
-```</t>
+          <t>Use np.linalg.norm(s1 - s2).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>astype() for type conversion</t>
+          <t>Visualization</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>- Convert columns to target dtypes.
-Example:
-```
-df['age'] = df['age'].astype('int64')
-```</t>
+          <t>df.plot, hist, boxplot for quick charts.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Merge and expand interview sections
Co-authored-by: impalalogis <impalalogis@gmail.com>
</commit_message>
<xml_diff>
--- a/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
+++ b/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
@@ -19,14 +19,12 @@
     <sheet name="Section J - Databricks" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Section K - Migration" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Section L - System Design" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Section M - SQL Practice" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Section N - PySpark Practice" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Section O - Databricks Jobs" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Section P - Behavioral" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Section Q - Arch Visuals" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Section R - Mock QA" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Section H - Spark Optimization" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Section S - Cloud Map" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Section O - Databricks Jobs" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Section P - Behavioral" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Section Q - Arch Visuals" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Section R - Mock QA" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Section H - Spark Optimization" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Section S - Cloud Map" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1052,144 +1050,144 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Auto Loader</t>
+          <t>Lakehouse | Delta Lake basics</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Incremental file ingestion with schema inference and evolution.</t>
+          <t>Delta provides ACID, schema enforcement, and time travel on cloud storage. This enables reliable batch and streaming.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Delta Lake</t>
+          <t>Lakehouse | Medallion architecture</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ACID tables with schema enforcement and time travel.</t>
+          <t>Explain Bronze for raw, Silver for cleaned, Gold for curated. This improves lineage and reusability.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Medallion architecture</t>
+          <t>Lakehouse | Auto Loader</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bronze raw, Silver cleansed, Gold curated.</t>
+          <t>Incremental ingestion with schema inference and evolution. Use for scalable file discovery.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jobs and Workflows</t>
+          <t>Lakehouse | Delta Live Tables</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Schedule tasks with dependencies, retries, and alerts.</t>
+          <t>Managed pipelines with declarative transformations and built-in quality checks. Useful for standard ETL.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cluster types</t>
+          <t>Compute | Cluster types</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>All-purpose for dev; job clusters for production.</t>
+          <t>All-purpose for dev, job clusters for production. Job clusters reduce cost and improve isolation.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Unity Catalog</t>
+          <t>Compute | Photon engine</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Centralized governance for data, permissions, and lineage.</t>
+          <t>Vectorized engine for faster SQL and Delta queries. Highlight when performance gains are most visible.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Databricks SQL</t>
+          <t>Compute | Caching strategy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SQL warehouses for BI and ad-hoc analytics.</t>
+          <t>Cache reused DataFrames and unpersist after use. Avoid caching large single-use datasets.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Photon engine</t>
+          <t>Compute | OPTIMIZE and Z-ORDER</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vectorized engine for faster SQL/Delta.</t>
+          <t>Compact small files and improve data skipping. Emphasize selective query performance.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Delta Live Tables</t>
+          <t>Governance | Unity Catalog</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Managed pipelines with declarative transformations.</t>
+          <t>Centralized permissions, data discovery, and lineage. Enforce access by groups and domains.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MLflow basics</t>
+          <t>Governance | Secrets management</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Track experiments and manage model registry.</t>
+          <t>Use secret scopes for credentials and rotate regularly. Avoid hard-coding secrets in notebooks.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Repos and versioning</t>
+          <t>Governance | Repos and CI/CD</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Git-backed notebooks and code collaboration.</t>
+          <t>Git-backed repos allow code review and promotion. Automate deployments via pipelines.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Secrets management</t>
+          <t>MLOps | MLflow basics</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Use secret scopes to store credentials.</t>
+          <t>Track experiments, log metrics, and manage model registry. Enables reproducible ML workflows.</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1452,180 +1450,144 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Batch architecture</t>
+          <t>Batch/Lakehouse | Batch ETL design</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Scheduled ETL optimized for throughput and cost.</t>
+          <t>Describe source ingestion, staging, transforms, and curated outputs. Emphasize idempotency and partitioning.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Streaming architecture</t>
+          <t>Batch/Lakehouse | Lakehouse architecture</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Low-latency ingestion with checkpointing and watermarking.</t>
+          <t>Combine data lake storage with warehouse governance. Use Bronze/Silver/Gold and Delta for ACID.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lambda vs Kappa</t>
+          <t>Batch/Lakehouse | Data modeling and grain</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lambda uses batch + stream; Kappa uses stream only.</t>
+          <t>Define grain before dimensions and facts. This prevents aggregation errors later.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lakehouse architecture</t>
+          <t>Batch/Lakehouse | Partitioning strategy</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Data lake storage with warehouse-style governance and performance.</t>
+          <t>Partition by high-cardinality keys or time for pruning. Avoid over-partitioning small files.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Event-driven pipelines</t>
+          <t>Streaming | Real-time pipeline</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Use events/queues to trigger processing.</t>
+          <t>Use Structured Streaming with checkpoints and watermarking. Handle late data and exactly-once semantics.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Data quality layers</t>
+          <t>Streaming | Lambda vs Kappa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Validate in Silver and quarantine bad records.</t>
+          <t>Lambda uses batch + stream; Kappa uses stream-only. Pick based on operational complexity.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Metadata and lineage</t>
+          <t>Streaming | CDC design</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Catalog schemas, ownership, and data lineage.</t>
+          <t>Capture changes, dedupe with windows, and MERGE into targets. Maintain audit columns.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>High availability and failover</t>
+          <t>Streaming | Backpressure handling</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Multi-AZ, retries, and resilient storage.</t>
+          <t>Use rate limits and autoscaling. Monitor lag and tune micro-batch intervals.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Orchestration patterns</t>
+          <t>Governance | Data quality framework</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DAG-based dependencies and idempotent tasks.</t>
+          <t>Rule-driven checks with quarantine and audit logs. Fail fast on critical rules.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Data modeling best practices</t>
+          <t>Governance | Lineage and catalog</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Define grain, keys, and dimensions early.</t>
+          <t>Register schemas, owners, and lineage for impact analysis. Improves compliance.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Design a real-time streaming pipeline</t>
+          <t>Governance | High availability</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ingest events, apply transformations, and write to Delta with checkpoints.</t>
+          <t>Use multi-AZ storage, retries, and failover clusters. Design for graceful degradation.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Design a data lakehouse</t>
+          <t>Governance | Cost optimization</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ADLS + Delta + governance; expose Gold tables to BI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Design a scalable ETL framework</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Metadata-driven configs and reusable transforms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Design a CDC pipeline</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Capture changes, dedupe, and MERGE into targets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Design a data quality framework</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Rule-driven checks with audit logs and quarantine.</t>
+          <t>Use incremental loads, autoscaling, and right-sized clusters. Optimize file sizes to reduce scan cost.</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1658,120 +1620,144 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Find the second highest salary</t>
+          <t>Design | Job types</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Use MAX with subquery or DENSE_RANK = 2.</t>
+          <t>Notebook, Python, JAR, and SQL tasks are supported. Choose based on codebase and runtime needs.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Get duplicate rows</t>
+          <t>Design | Job clusters vs all-purpose</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GROUP BY columns and HAVING COUNT(*) &gt; 1.</t>
+          <t>Job clusters are ephemeral and cost-efficient; all-purpose are interactive for development.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Employees earning more than managers</t>
+          <t>Design | Task orchestration</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Self-join employee to manager and compare salary.</t>
+          <t>Use task dependencies for DAG-style execution. Keep tasks small and idempotent.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Top N records</t>
+          <t>Design | Parameters and widgets</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ORDER BY metric DESC and LIMIT N.</t>
+          <t>Pass parameters via job inputs or widgets. This enables reusable pipelines.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Count per department</t>
+          <t>Ops | Scheduling</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GROUP BY department_id and COUNT(*).</t>
+          <t>Use cron or periodic schedules and align to SLAs. Avoid overlapping runs when not supported.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nth highest salary</t>
+          <t>Ops | Retry and timeout strategy</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Use DENSE_RANK over salary DESC.</t>
+          <t>Set retries with backoff and timeouts per task. Fail fast on non-retriable errors.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Highest salary per department</t>
+          <t>Ops | Monitoring and alerting</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RANK or MAX with GROUP BY.</t>
+          <t>Use job notifications, logs, and dashboards. Route alerts to on-call channels.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Running total</t>
+          <t>Ops | Environment separation</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SUM over window ordered by time.</t>
+          <t>Separate dev/test/prod with configs and permissions. Use workspace or catalog isolation.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Find missing IDs</t>
+          <t>Security | Secrets in jobs</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Generate range and left join to find gaps.</t>
+          <t>Store credentials in secret scopes and reference them securely. Never embed secrets in code.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LEAD/LAG usage</t>
+          <t>Security | Service principals</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Use LAG/LEAD to access previous/next row.</t>
+          <t>Use service principals for automated jobs. Grant least-privilege access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Deployment | CI/CD for jobs</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Automate job creation and updates via pipelines. Keep job configs in version control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Deployment | Rollback strategy</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Revert job config and code to last stable version. Use Delta time travel if needed.</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1804,120 +1790,144 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Read CSV with schema</t>
+          <t>Leadership | Tell me about yourself</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>spark.read.schema(...).csv(path).</t>
+          <t>Provide a 60-second summary of experience, impact, and current focus. End with why the role fits.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Filter and select columns</t>
+          <t>Leadership | Biggest project you led</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>df.filter('x &gt; 10').select('a','b').</t>
+          <t>Highlight scope, stakeholders, and metrics. Focus on outcomes and lessons learned.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Join two DataFrames</t>
+          <t>Leadership | Conflict with stakeholder</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>df1.join(df2, on='id', how='left').</t>
+          <t>Explain the disagreement, how you aligned on priorities, and the compromise achieved.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GroupBy aggregate</t>
+          <t>Execution | Production incident</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>df.groupBy('dept').agg({'salary':'avg'}).</t>
+          <t>Use STAR: what broke, how you mitigated, and what you fixed permanently.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Window rank</t>
+          <t>Execution | Handling tight deadlines</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Use Window.partitionBy and rank over orderBy.</t>
+          <t>Describe prioritization, scope reduction, and communication cadence.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Handle nulls</t>
+          <t>Execution | Process improvement</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Use na.fill, na.drop, or coalesce.</t>
+          <t>Show how you automated a bottleneck and quantify the time saved.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Write Delta table</t>
+          <t>Growth | Weakness question</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>df.write.format('delta').saveAsTable('db.tbl').</t>
+          <t>Share a real weakness and the steps you took to improve.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Broadcast join</t>
+          <t>Growth | Failure you learned from</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Use broadcast() for small dimension tables.</t>
+          <t>Describe the failure, impact, and what you changed afterward.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cache and count</t>
+          <t>Growth | Mentoring juniors</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>df.cache(); df.count() to materialize.</t>
+          <t>Explain how you pair, review code, and give ownership with guidance.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Use spark.sql</t>
+          <t>Leadership | Leadership style</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Create temp view and run spark.sql query.</t>
+          <t>Describe how you balance autonomy, accountability, and support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Execution | Managing priorities</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Use impact vs effort and align with business goals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Leadership | Cross-team collaboration</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Show how you coordinate dependencies and keep decisions documented.</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1950,144 +1960,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Job types</t>
+          <t>Ingestion | Batch pipeline diagram</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Notebook, Python, JAR, SQL tasks are supported.</t>
+          <t>Show sources, ingestion, staging, and curated layers. Emphasize partitioning and error handling.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Job clusters vs all-purpose</t>
+          <t>Ingestion | Streaming pipeline diagram</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Job clusters are ephemeral; all-purpose are interactive.</t>
+          <t>Show event source, streaming ingestion, checkpoints, and Delta sinks. Mention watermarking.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Task orchestration</t>
+          <t>Processing | Lakehouse layers</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Define dependencies and run tasks in order.</t>
+          <t>Visualize Bronze/Silver/Gold with Delta and governance. Explain how data moves across layers.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Parameters and widgets</t>
+          <t>Processing | Serving layer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Pass parameters via job inputs or widgets.</t>
+          <t>Show BI or API access on Gold tables. Mention caching or SQL warehouses.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>DevOps | CI/CD flow</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Use cron or periodic schedules.</t>
+          <t>Diagram source control, build/test, and deployment stages. Include approval gates.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADF/Airflow integration</t>
+          <t>DevOps | Monitoring layer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Trigger Databricks jobs via REST API.</t>
+          <t>Include logs, metrics, and alerting for pipelines. Show how failures are triaged.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Environments</t>
+          <t>Migration | Cutover diagram</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Separate dev/test/prod with configs and permissions.</t>
+          <t>Show parallel runs, validation checks, and final cutover. Include rollback path.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Alerting and monitoring</t>
+          <t>Migration | Data validation steps</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Use job notifications and logs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Retry and timeout strategy</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Configure retries, backoff, and timeouts per task.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Secrets in jobs</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Store credentials in secret scopes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Deployment via CI/CD</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Automate job creation and updates via pipelines.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Rollback of jobs</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Revert job config and code to last stable version.</t>
+          <t>Show row counts, checksums, and business KPI reconciliation.</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2120,156 +2082,240 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tell me about yourself</t>
+          <t>Databricks | What is Delta Lake?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Summarize experience, impact, and current focus in 60 seconds.</t>
+          <t>Delta adds ACID transactions, schema enforcement, and time travel on cloud storage. It reduces data corruption and enables reliable pipelines.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Biggest project you led</t>
+          <t>Databricks | When to use Auto Loader?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Highlight scope, stakeholders, and measurable outcomes.</t>
+          <t>Use Auto Loader for incremental file ingestion at scale. It handles schema evolution and efficient file discovery.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Production incident</t>
+          <t>Databricks | Explain Unity Catalog</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Use STAR: what failed, how you fixed it, and prevention.</t>
+          <t>Unity Catalog centralizes governance for data, permissions, and lineage. It enables consistent access controls across workspaces.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Conflict with stakeholder</t>
+          <t>Databricks | What is Photon?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Show alignment, tradeoffs, and a phased compromise.</t>
+          <t>Photon is a vectorized execution engine for faster SQL and Delta workloads. It helps with BI and large scans.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mentoring juniors</t>
+          <t>Databricks | Delta OPTIMIZE vs VACUUM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pairing, code reviews, and clear learning goals.</t>
+          <t>OPTIMIZE compacts small files for faster reads. VACUUM removes obsolete files to reduce storage and metadata.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Handling tight deadlines</t>
+          <t>Spark | RDD vs DataFrame vs Dataset</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Prioritize critical scope and communicate early.</t>
+          <t>RDD is low-level and flexible; DataFrame is optimized and schema-based; Dataset adds types in Scala/Java.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Weakness question</t>
+          <t>Spark | What causes shuffles?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Be honest and show improvement steps.</t>
+          <t>Wide transformations like join, groupBy, and distinct trigger shuffles. They are expensive and should be minimized.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Why this role/company</t>
+          <t>Spark | How to handle skew?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Connect skills to role needs and mission.</t>
+          <t>Use salting, broadcast joins, or range partitioning. Validate improvements in Spark UI.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Failure you learned from</t>
+          <t>Spark | Explain AQE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Explain lesson and process change.</t>
+          <t>Adaptive Query Execution adjusts joins, skew, and partitions at runtime. It improves stability and performance.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Leadership style</t>
+          <t>Spark | Cache vs persist</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Supportive, data-driven, and accountable.</t>
+          <t>Cache uses memory by default; persist allows different storage levels. Use when datasets are reused.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Process improvement</t>
+          <t>SQL | Difference between RANK and DENSE_RANK</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Automate bottlenecks and measure gains.</t>
+          <t>RANK leaves gaps after ties; DENSE_RANK does not. Choose based on reporting needs.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Managing priorities</t>
+          <t>SQL | Find duplicates</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Use impact vs effort and stakeholder alignment.</t>
+          <t>GROUP BY columns and HAVING COUNT(*) &gt; 1 identifies duplicates. Join back to get full rows.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cross-team collaboration</t>
+          <t>SQL | Nth highest salary</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Regular syncs and clear documentation.</t>
+          <t>Use DENSE_RANK over salary DESC and filter rnk = N. Handles ties correctly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SQL | Window functions use cases</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Running totals, ranking, and lag/lead comparisons. They avoid complex self-joins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SQL | How to compare two tables</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Use FULL OUTER JOIN or EXCEPT/UNION to detect mismatches. Validate on key columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Databricks | CDC pipeline design</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ingest changes, dedupe by key/time, then MERGE into Delta. Maintain audit columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Spark | Optimize slow job</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Profile stages, fix skew, prune columns, tune partitions, and cache reused data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Governance | How do you handle PII?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Mask or tokenize sensitive fields and restrict access with RBAC. Log access for audits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Reliability | How to rollback bad release?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Revert code, restore Delta tables with time travel, and rerun affected jobs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Modeling | Fact vs dimension</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Facts store measures and foreign keys; dimensions store descriptive attributes. Grain is critical.</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2302,60 +2348,516 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lakehouse</t>
+          <t>Driver, executors, cluster manager</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bronze/Silver/Gold layers on Delta with governance.</t>
+          <t>Driver schedules work; executors run tasks; manager allocates resources.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Batch ingestion</t>
+          <t>RDD vs DataFrame vs Dataset</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Scheduled loads into raw then curated layers.</t>
+          <t>RDD is low-level; DataFrame is optimized; Dataset is typed (Scala/Java).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>Lazy evaluation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Real-time ingestion with checkpoints and watermarking.</t>
+          <t>Transforms build a DAG; actions trigger execution.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CI/CD</t>
+          <t>Transformations vs actions</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Source control, build, test, deploy pipeline.</t>
+          <t>Transformations create lineage; actions materialize results.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Narrow vs wide transformations</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Parallel run, validation, and controlled cutover.</t>
+          <t>Narrow avoids shuffle; wide causes shuffle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Catalyst optimizer</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Optimizes logical and physical plans for SQL/DataFrames.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tungsten engine</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Uses codegen and binary processing for performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Shuffle mechanics</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Shuffle moves data across partitions and is expensive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Broadcast joins</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Broadcast small tables to avoid shuffle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Broadcast hint</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Force broadcast when auto-broadcast does not trigger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Caching and persisting</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cache reused DataFrames; unpersist when done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Partitioning strategy</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Partition by high-cardinality keys for parallelism, low-cardinality for pruning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Repartition vs coalesce</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Repartition balances with shuffle; coalesce reduces partitions without shuffle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AQE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Adaptive Query Execution tunes joins, skew, and partitions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Shuffle partitions tuning</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Adjust spark.sql.shuffle.partitions to cluster size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Skew handling</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Use salting, range partitioning, or broadcast to fix skew.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Predicate pushdown</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Push filters to source to reduce scan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Column pruning</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Select only required columns to save memory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Avoid Python UDFs</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Prefer built-in functions or pandas UDFs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Avoid wide transformations</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Filter early and pre-aggregate to reduce shuffles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>mapPartitions vs map</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Process batches per partition for efficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Avoid collect()</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Do not bring large data to driver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Avoid explode on large arrays</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Explode can cause huge shuffles; pre-filter arrays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Window functions</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Partition wisely; window ops can shuffle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>File size tuning</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Target 128-512 MB files to avoid small-file overhead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Delta OPTIMIZE</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Compact small files to improve reads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Z-ORDER</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Co-locate data to improve selective query skipping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Data skipping stats</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Delta stores min/max stats for pruning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Bloom filters</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Speed up selective joins and lookups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Delta MERGE</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Use MERGE for upserts and SCD handling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Delta CDF</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Use Change Data Feed for incremental processing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Auto Loader</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Incremental ingestion with schema evolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Auto-Optimize / Optimize Write</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Auto-compact files during writes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>VACUUM</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Remove obsolete files to reduce metadata and storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Liquid clustering</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Next-gen clustering for large Delta tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Photon engine</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Vectorized engine for faster SQL/Delta on Databricks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Avoid cross joins</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Cross joins explode data unless required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Incremental ETL</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Process only changes to reduce cost and latency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Range partitioning for time-series</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Partition by date for pruning and parallelism.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Checkpointing</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Break long lineage and improve stability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Avoid repeated reads</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Cache or checkpoint to reuse datasets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Use explain()</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Inspect plans to spot expensive stages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Cluster sizing and autoscaling</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Right-size executors and use autoscaling for peak loads.</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2388,722 +2890,168 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RDD vs DataFrame vs Dataset</t>
+          <t>CI/CD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RDD is low-level; DataFrame is optimized; Dataset is typed (Scala/Java).</t>
+          <t>CDP: Bitbucket/Jenkins/RLM; Azure: Azure DevOps/GitHub; AWS: CodeBuild/CodeDeploy/CodePipeline; GCP: Cloud Build/Cloud Deploy.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Handle skew in Spark</t>
+          <t>Data Warehouse</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Use salting, broadcast joins, or range partitioning.</t>
+          <t>CDP: Hive/Impala; Azure: Synapse; AWS: Redshift; GCP: BigQuery.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Z-ORDER in Delta</t>
+          <t>Data Integration</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Improves data skipping by co-locating values.</t>
+          <t>CDP: PySpark/NiFi/Sqoop; Azure: Data Factory; AWS: Glue/Data Pipeline; GCP: Data Fusion.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Design CDC pipeline</t>
+          <t>Messaging</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Capture changes, dedupe, MERGE to target.</t>
+          <t>CDP: JMS/Kafka; Azure: Service Bus/Event Hubs; AWS: Kinesis/SNS/SQS; GCP: Pub/Sub.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ensure data quality</t>
+          <t>Workflow Orchestration</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Define rules, apply in Spark, quarantine failures.</t>
+          <t>CDP: Oozie/Autosys/Airflow; Azure: Data Factory/Logic Apps; AWS: Step Functions/Glue Workflows; GCP: Composer.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>What is Delta Lake</t>
+          <t>Document DB</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ACID tables with schema enforcement and time travel.</t>
+          <t>CDP: N/A or HBase; Azure: Cosmos DB; AWS: DocumentDB; GCP: Firestore.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Auto Loader use case</t>
+          <t>NoSQL (Key/Value)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Incremental file ingestion with schema evolution.</t>
+          <t>CDP: HBase; Azure: Cosmos DB; AWS: DynamoDB; GCP: Bigtable.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>When to broadcast join</t>
+          <t>RDBMS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>When one table is small enough to fit in memory.</t>
+          <t>CDP: Hive/Impala/Oracle; Azure: Azure SQL Database; AWS: Aurora/RDS; GCP: Cloud SQL.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Difference between RANK and DENSE_RANK</t>
+          <t>Storage Transfer</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>RANK leaves gaps; DENSE_RANK does not.</t>
+          <t>CDP: DistCp/NiFi; Azure: Data Factory/Storage Mover; AWS: Storage Gateway/DataSync; GCP: Storage Transfer Service.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Find duplicates in SQL</t>
+          <t>Network Connectivity</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GROUP BY and HAVING COUNT(*) &gt; 1.</t>
+          <t>CDP: Knox/SDX; Azure: VPN Gateway; AWS: VPN; GCP: Cloud VPN.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nth highest salary</t>
+          <t>Audit Logging</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Use DENSE_RANK over salary DESC.</t>
+          <t>CDP: Ranger Audit/Cloudera Navigator; Azure: Monitor/Audit Logs; AWS: CloudTrail; GCP: Cloud Audit Logs.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Spark shuffle triggers</t>
+          <t>Key Management</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Wide transformations like join, groupBy, distinct.</t>
+          <t>CDP: CyberArk/Ranger KMS; Azure: Key Vault; AWS: KMS; GCP: Cloud KMS.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Optimize slow Spark job</t>
+          <t>Identity Management</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Profile stages, fix skew, tune partitions, cache reuse.</t>
+          <t>CDP: LDAP/Sentry/Ranger; Azure: Active Directory; AWS: IAM; GCP: Cloud IAM.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Handle PII data</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Mask/encrypt and enforce RBAC with audits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Rollback bad release</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Revert code and restore Delta tables via time travel.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B44"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Driver, executors, cluster manager</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Driver schedules work; executors run tasks; manager allocates resources.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>RDD vs DataFrame vs Dataset</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RDD is low-level; DataFrame is optimized; Dataset is typed (Scala/Java).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Lazy evaluation</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Transforms build a DAG; actions trigger execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Transformations vs actions</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Transformations create lineage; actions materialize results.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Narrow vs wide transformations</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Narrow avoids shuffle; wide causes shuffle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Catalyst optimizer</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Optimizes logical and physical plans for SQL/DataFrames.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Tungsten engine</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Uses codegen and binary processing for performance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Shuffle mechanics</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Shuffle moves data across partitions and is expensive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Broadcast joins</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Broadcast small tables to avoid shuffle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Broadcast hint</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Force broadcast when auto-broadcast does not trigger.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Caching and persisting</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Cache reused DataFrames; unpersist when done.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Partitioning strategy</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Partition by high-cardinality keys for parallelism, low-cardinality for pruning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Repartition vs coalesce</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Repartition balances with shuffle; coalesce reduces partitions without shuffle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>AQE</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Adaptive Query Execution tunes joins, skew, and partitions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Shuffle partitions tuning</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Adjust spark.sql.shuffle.partitions to cluster size.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Skew handling</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Use salting, range partitioning, or broadcast to fix skew.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Predicate pushdown</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Push filters to source to reduce scan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Column pruning</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Select only required columns to save memory.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Avoid Python UDFs</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Prefer built-in functions or pandas UDFs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Avoid wide transformations</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Filter early and pre-aggregate to reduce shuffles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>mapPartitions vs map</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Process batches per partition for efficiency.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Avoid collect()</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Do not bring large data to driver.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Avoid explode on large arrays</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Explode can cause huge shuffles; pre-filter arrays.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Window functions</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Partition wisely; window ops can shuffle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>File size tuning</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Target 128-512 MB files to avoid small-file overhead.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Delta OPTIMIZE</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Compact small files to improve reads.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Z-ORDER</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Co-locate data to improve selective query skipping.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Data skipping stats</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Delta stores min/max stats for pruning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Bloom filters</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Speed up selective joins and lookups.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Delta MERGE</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Use MERGE for upserts and SCD handling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Delta CDF</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Use Change Data Feed for incremental processing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Auto Loader</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Incremental ingestion with schema evolution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Auto-Optimize / Optimize Write</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Auto-compact files during writes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>VACUUM</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Remove obsolete files to reduce metadata and storage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Liquid clustering</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Next-gen clustering for large Delta tables.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Photon engine</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Vectorized engine for faster SQL/Delta on Databricks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Avoid cross joins</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Cross joins explode data unless required.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Incremental ETL</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Process only changes to reduce cost and latency.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Range partitioning for time-series</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Partition by date for pruning and parallelism.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Checkpointing</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Break long lineage and improve stability.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Avoid repeated reads</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Cache or checkpoint to reuse datasets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Use explain()</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Inspect plans to spot expensive stages.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Cluster sizing and autoscaling</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Right-size executors and use autoscaling for peak loads.</t>
+          <t>CDP: HDFS; Azure: ADLS Gen2; AWS: S3; GCP: Cloud Storage.</t>
         </is>
       </c>
     </row>
@@ -3322,200 +3270,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CI/CD</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>CDP: Bitbucket/Jenkins/RLM; Azure: Azure DevOps/GitHub; AWS: CodeBuild/CodeDeploy/CodePipeline; GCP: Cloud Build/Cloud Deploy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Data Warehouse</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CDP: Hive/Impala; Azure: Synapse; AWS: Redshift; GCP: BigQuery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Data Integration</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>CDP: PySpark/NiFi/Sqoop; Azure: Data Factory; AWS: Glue/Data Pipeline; GCP: Data Fusion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Messaging</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>CDP: JMS/Kafka; Azure: Service Bus/Event Hubs; AWS: Kinesis/SNS/SQS; GCP: Pub/Sub.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Workflow Orchestration</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CDP: Oozie/Autosys/Airflow; Azure: Data Factory/Logic Apps; AWS: Step Functions/Glue Workflows; GCP: Composer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Document DB</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CDP: N/A or HBase; Azure: Cosmos DB; AWS: DocumentDB; GCP: Firestore.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>NoSQL (Key/Value)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>CDP: HBase; Azure: Cosmos DB; AWS: DynamoDB; GCP: Bigtable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>RDBMS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CDP: Hive/Impala/Oracle; Azure: Azure SQL Database; AWS: Aurora/RDS; GCP: Cloud SQL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Storage Transfer</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CDP: DistCp/NiFi; Azure: Data Factory/Storage Mover; AWS: Storage Gateway/DataSync; GCP: Storage Transfer Service.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Network Connectivity</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CDP: Knox/SDX; Azure: VPN Gateway; AWS: VPN; GCP: Cloud VPN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Audit Logging</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>CDP: Ranger Audit/Cloudera Navigator; Azure: Monitor/Audit Logs; AWS: CloudTrail; GCP: Cloud Audit Logs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Key Management</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CDP: CyberArk/Ranger KMS; Azure: Key Vault; AWS: KMS; GCP: Cloud KMS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Identity Management</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>CDP: LDAP/Sentry/Ranger; Azure: Active Directory; AWS: IAM; GCP: Cloud IAM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>CDP: HDFS; Azure: ADLS Gen2; AWS: S3; GCP: Cloud Storage.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4215,7 +3969,8 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Use pd.DataFrame or pd.Series from list, dict, or array.</t>
+          <t>Create from list/dict/array.
+Example: pd.DataFrame({"name": ["A"], "age": [30]}).</t>
         </is>
       </c>
     </row>
@@ -4227,7 +3982,8 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>read_csv/read_excel; to_csv/to_excel; set encoding if needed.</t>
+          <t>Use pandas readers and writers.
+Example: df = pd.read_csv("file.csv"); df.to_excel("out.xlsx", index=False).</t>
         </is>
       </c>
     </row>
@@ -4239,7 +3995,8 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>head, tail, info, describe, shape for quick profiling.</t>
+          <t>Quick profiling with head/info/describe.
+Example: df.head(); df.info(); df.describe().</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4008,8 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>dtypes, astype, to_numeric, to_datetime.</t>
+          <t>Convert with astype or to_datetime.
+Example: df["dt"] = pd.to_datetime(df["dt"]).</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4021,8 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>loc/at label-based; iloc/iat position-based.</t>
+          <t>Label vs position access.
+Example: df.loc[5, "name"]; df.iloc[0, 1].</t>
         </is>
       </c>
     </row>
@@ -4275,7 +4034,8 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Boolean masks, query(), isin(), between().</t>
+          <t>Boolean masks or query.
+Example: df[df["salary"] &gt; 100000].</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4047,8 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>isnull/notnull, fillna, dropna.</t>
+          <t>Detect and fill/drop missing data.
+Example: df.fillna({"city": "Unknown"}).</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4060,8 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>duplicated and drop_duplicates; columns via df.columns.duplicated.</t>
+          <t>Find and drop duplicates.
+Example: df.drop_duplicates(subset=["id"]).</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4073,8 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>sort_values/sort_index; nlargest/nsmallest for top/bottom.</t>
+          <t>Sort rows and pick top N.
+Example: df.sort_values("salary", ascending=False).head(5).</t>
         </is>
       </c>
     </row>
@@ -4323,7 +4086,8 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>reindex aligns labels; reset_index moves index to column.</t>
+          <t>Reindex aligns labels; reset_index makes index a column.
+Example: df.reset_index(drop=True).</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4099,8 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>groupby keys, agg metrics; transform returns aligned output.</t>
+          <t>Group and aggregate metrics.
+Example: df.groupby("dept").agg({"salary": "mean"}).</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4112,8 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>merge on keys, join on index, concat rows or columns.</t>
+          <t>Combine dataframes by keys or index.
+Example: df1.merge(df2, on="id", how="left").</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4125,8 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pivot_table for aggregates; crosstab for counts.</t>
+          <t>Summarize to matrix form.
+Example: pd.pivot_table(df, index="dept", values="salary", aggfunc="mean").</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4138,8 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Use Series.str methods like lower, contains, replace.</t>
+          <t>Use vectorized string methods.
+Example: df["email"].str.contains("@").</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4151,8 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>to_datetime, dt accessor, resample, shift.</t>
+          <t>Use dt accessor and resample.
+Example: df.set_index("dt").resample("M").sum().</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4164,8 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>map for Series; apply for rows/cols; applymap elementwise.</t>
+          <t>Map for Series; apply for rows.
+Example: df["score"].map(lambda x: x * 2).</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4177,8 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>replace values; clip bounds outliers.</t>
+          <t>Replace values or clip bounds.
+Example: df["pct"].clip(0, 100).</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4190,8 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Use df.copy() to avoid chained assignment side effects.</t>
+          <t>Copy to avoid chained assignment issues.
+Example: df_copy = df.copy().</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4203,8 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>df.empty is True when no rows or columns.</t>
+          <t>Use df.empty to validate content.
+Example: if df.empty: ...</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4216,8 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>df.iloc[::-1].reset_index(drop=True).</t>
+          <t>Reverse and reset index.
+Example: df.iloc[::-1].reset_index(drop=True).</t>
         </is>
       </c>
     </row>
@@ -4455,7 +4229,8 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Use isin to keep values not present in the other Series.</t>
+          <t>Keep values not in the other series.
+Example: s1[~s1.isin(s2)].</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4242,8 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Use value_counts().nlargest(N) to keep top values.</t>
+          <t>Keep top values and replace rest.
+Example: top = s.value_counts().nlargest(2).index.</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4255,8 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Filter with s[s % k == 0] for divisibility.</t>
+          <t>Filter by divisibility.
+Example: s[s % 3 == 0].</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4268,8 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Use np.linalg.norm(s1 - s2).</t>
+          <t>Compute with numpy.
+Example: np.linalg.norm(s1 - s2).</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4281,8 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>df.plot, hist, boxplot for quick charts.</t>
+          <t>Quick charts with plot/hist/boxplot.
+Example: df["age"].hist().</t>
         </is>
       </c>
     </row>
@@ -4518,7 +4297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4540,96 +4319,194 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SQL vs PySpark equivalents</t>
+          <t>Read CSV with schema</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DataFrame API mirrors SQL: select, filter, groupBy, join.</t>
+          <t>Use an explicit schema to avoid type drift.
+Example: df = spark.read.schema(schema).csv(path).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>String functions</t>
+          <t>Filter and select columns</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Use pyspark.sql.functions like upper, lower, concat, regexp_replace.</t>
+          <t>Use filter and select for projection and predicates.
+Example: df.filter("x &gt; 10").select("a", "b").</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Date functions</t>
+          <t>Join two DataFrames</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Use datediff, date_add/sub, date_format, current_date.</t>
+          <t>Join on keys with the right join type.
+Example: df1.join(df2, on="id", how="left").</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Window functions</t>
+          <t>GroupBy aggregate</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Define Window partition/order and apply rank, sum, lag/lead.</t>
+          <t>Aggregate with groupBy and agg.
+Example: df.groupBy("dept").agg({"salary": "avg"}).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Temp views and spark.sql</t>
+          <t>Window rank</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>createOrReplaceTempView then query with spark.sql.</t>
+          <t>Use Window to rank within partitions.
+Example: rank().over(Window.partitionBy("dept").orderBy(col("salary").desc())).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Write and read tables</t>
+          <t>Handle nulls</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>df.write.saveAsTable and spark.read.table.</t>
+          <t>Use na.fill, na.drop, or coalesce.
+Example: df.na.fill({"city": "Unknown"}).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Drop duplicates</t>
+          <t>Write Delta table</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>dropDuplicates on all or selected columns.</t>
+          <t>Write to Delta for ACID and time travel.
+Example: df.write.format("delta").saveAsTable("db.tbl").</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Broadcast join</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Broadcast small dimensions to avoid shuffle.
+Example: df.join(broadcast(dim), "id").</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cache and count</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cache reused dataframes and materialize once.
+Example: df.cache(); df.count().</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Temp view and spark.sql</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Query DataFrames with SQL when convenient.
+Example: df.createOrReplaceTempView("t"); spark.sql("SELECT * FROM t").</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>String functions</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Use built-in functions for string cleanup.
+Example: df.select(F.upper("name"), F.regexp_replace("name", " ", "_"))).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Date functions</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Use datediff/date_add/date_format for date logic.
+Example: df.select(F.date_add("dt", 7)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Casting columns</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Use col.cast or withColumn to change types.</t>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cast to target types explicitly.
+Example: df.withColumn("amt", F.col("amt").cast("double")).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Drop duplicates</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Remove duplicates by all or selected columns.
+Example: df.dropDuplicates(["id"]).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UDF vs built-in functions</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Prefer built-ins for performance; use UDFs only when needed.</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4666,120 +4543,144 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Azure Data Factory pipelines</t>
+          <t>Platform | Warehouse choices</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Orchestrate data movement with linked services, datasets, and triggers.</t>
+          <t>Explain trade-offs: Redshift and Synapse are warehouse-first; BigQuery is serverless and scales per query. Tie selection to workload, cost model, and latency needs.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Databricks notebooks and Delta</t>
+          <t>Platform | Storage layer</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Notebooks for Spark; Delta adds ACID, schema, time travel.</t>
+          <t>Compare ADLS, S3, GCS for durability, cost, and integration. Mention partitioning strategy and lifecycle policies.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Spark and PySpark transformations</t>
+          <t>Platform | Databricks vs native warehouse</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Transformations are lazy; actions trigger execution.</t>
+          <t>Choose Databricks for Spark/Delta and ML workloads; choose native warehouse for pure BI analytics. Highlight interoperability when both are used.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hadoop, HDFS, Hive</t>
+          <t>Integration | ETL tool selection</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hadoop ecosystem; HDFS storage; Hive provides SQL on HDFS.</t>
+          <t>ADF, Glue, and Data Fusion all orchestrate ingestion; choose based on cloud footprint and connector needs. Note cost, integration, and monitoring features.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kafka basics</t>
+          <t>Integration | Orchestration strategy</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Distributed log with topics, partitions, producers, consumers.</t>
+          <t>Airflow provides portable DAGs; ADF provides managed pipelines in Azure. Discuss retries, SLA alerts, and dependency handling.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CI/CD with Jenkins</t>
+          <t>Integration | Event streaming</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Automate build, test, deploy with Jenkinsfile pipelines.</t>
+          <t>Kafka/Kinesis/PubSub differ by managed depth and ecosystem. Emphasize ordering, partitions, and consumer lag monitoring.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Autosys/Airflow scheduling</t>
+          <t>Integration | CI/CD for data pipelines</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DAG-based orchestration with dependencies, retries, alerts.</t>
+          <t>Use Git-based workflows and automated tests for notebooks and SQL. Promote artifacts across environments with approvals.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Data quality checks</t>
+          <t>Governance | IAM and RBAC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Validate completeness, uniqueness, ranges, and referential integrity.</t>
+          <t>Use least privilege with service principals and group-based access. Tie to Unity Catalog or cloud IAM policies.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Data governance</t>
+          <t>Governance | Data catalog and lineage</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ownership, lineage, access control, PII handling.</t>
+          <t>Use catalog for schema ownership and lineage for auditability. This improves compliance and impact analysis.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>API development for ingestion</t>
+          <t>Governance | PII handling</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>REST endpoints with auth, pagination, validation, retries.</t>
+          <t>Apply masking, encryption, and access controls. Audit access and enforce data retention policies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Governance | Key management</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Use KMS/Key Vault and rotate secrets. Separate keys per environment for risk isolation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Governance | Data quality checks</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Implement null, range, and referential integrity checks in pipelines. Fail fast and quarantine bad records.</t>
         </is>
       </c>
     </row>
@@ -5086,7 +4987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5104,324 +5005,180 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Design end-to-end Databricks + ADF pipeline</t>
+          <t>Architecture | End-to-end ADF + Databricks pipeline</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ADF orchestrates, Databricks processes, Delta stores Bronze/Silver/Gold.</t>
+          <t>Describe ingestion with ADF, processing in Databricks, and Delta storage in Bronze/Silver/Gold. Emphasize idempotency and monitoring.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Design Lakehouse architecture</t>
+          <t>Architecture | Lakehouse design</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ADLS + Delta + governance with BI on Gold tables.</t>
+          <t>Use ADLS + Delta + Unity Catalog. Explain how governance and performance are balanced in the Gold layer.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Migrate Cloudera to Azure Databricks</t>
+          <t>Architecture | CDC ingestion</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Map services, migrate data, convert Hive to Delta, validate, cutover.</t>
+          <t>Capture changes, dedupe by key and timestamp, then MERGE into targets. Highlight late-arriving data handling.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Handle schema evolution in Delta Lake</t>
+          <t>Architecture | Schema evolution</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Use schema enforcement and evolution with controlled changes.</t>
+          <t>Enforce schema on write and allow controlled evolution with audits. Protect downstream consumers from breaking changes.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Design CDC ingestion</t>
+          <t>Architecture | Migration plan</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ingest changes, dedupe by key/timestamp, MERGE into target.</t>
+          <t>Map CDP services to Azure, migrate data, refactor jobs, validate, then cutover. Use parallel runs to reduce risk.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Build Medallion architecture</t>
+          <t>Performance | Reduce 3-hour Spark job</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bronze raw, Silver cleansed, Gold curated.</t>
+          <t>Profile stages, fix skew, prune columns, and tune partitions. Show before/after metrics to prove improvement.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Reduce 3-hour Spark job</t>
+          <t>Performance | Handle data skew</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Profile stages, fix skew, prune columns, tune partitions.</t>
+          <t>Use salting, broadcast joins, or range partitioning. Validate skew reduction in Spark UI.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Handle data skew</t>
+          <t>Performance | Reduce shuffles</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Use salting, broadcast joins, or range partitioning.</t>
+          <t>Avoid wide transformations and pre-aggregate early. Partition by join keys to minimize shuffle volume.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Optimize SQL queries</t>
+          <t>Performance | Cost optimization</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Filter early, avoid SELECT *, use proper indexing/partitioning.</t>
+          <t>Right-size clusters, use autoscaling, and optimize file sizes. Reduce recompute via caching and incremental loads.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Reduce shuffle operations</t>
+          <t>Reliability | Debug failing Spark jobs</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Minimize wide transforms and pre-aggregate.</t>
+          <t>Check driver/executor logs and the Spark UI. Reproduce with small samples and add data quality checks.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Optimize ADF pipelines</t>
+          <t>Reliability | Recover Delta tables</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Increase parallelism and offload heavy compute to Databricks.</t>
+          <t>Use time travel or restore from checkpoints. Explain how you validate data consistency post-recovery.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Implement data quality checks</t>
+          <t>Reliability | 2 AM pipeline failure</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Rule-based validation with quarantine for bad records.</t>
+          <t>Triage quickly, communicate impact, rerun with backfill, and add alerts to prevent repeat issues.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Enforce schema validation</t>
+          <t>Leadership | Mentor junior engineers</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Validate at ingestion and enforce Delta schema.</t>
+          <t>Use pairing, code reviews, and clear ownership. Tie feedback to measurable growth milestones.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Design audit logging</t>
+          <t>Leadership | Conflicting requirements</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Capture counts, timestamps, status, and lineage.</t>
+          <t>Align on priorities with stakeholders and deliver in phases. Provide a clear trade-off summary.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Handle PII data</t>
+          <t>Leadership | Communicate delays</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mask/encrypt and restrict access with RBAC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>CI/CD for Databricks notebooks</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Git-based repos and pipelines for promotion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Version control strategy</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Use feature branches, PRs, and tags.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Deployment automation</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Automate notebook/job deployment via CI/CD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Rollback strategy</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Revert code and use Delta time travel if needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Debug failing Spark jobs</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Use Spark UI, logs, and data checks to isolate cause.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Recover corrupted Delta tables</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Use time travel or restore from snapshot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Handle accidental deletes</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Restore with Delta time travel and enforce permissions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Manage 2 AM pipeline failures</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Triage, communicate, rerun with backfill, add alerts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Mentor junior engineers</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Pairing, reviews, and incremental ownership.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Handle conflicting requirements</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Prioritize with stakeholders and deliver in phases.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Communicate delays</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Share impact, revised timeline, and mitigation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Ensure cross-team alignment</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Regular syncs and documented decisions.</t>
+          <t>Share root cause, new timeline, and mitigation steps. Keep stakeholders updated until resolution.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consolidate Databricks/Azure interview Q&A
Co-authored-by: impalalogis <impalalogis@gmail.com>
</commit_message>
<xml_diff>
--- a/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
+++ b/Aniket_Singh_Senior_Data_Engineer_Interview_Prep.xlsx
@@ -12,19 +12,12 @@
     <sheet name="Section C - Python" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Section D - Pandas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Section E - PySpark" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Section F - Cloud" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Section 0 - Intro" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Section G - CI_CD" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Section I - Lead Scenarios" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Section J - Databricks" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Section K - Migration" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Section L - System Design" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Section O - Databricks Jobs" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Section P - Behavioral" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Section Q - Arch Visuals" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Section R - Mock QA" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Section H - Spark Optimization" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Section S - Cloud Map" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Section 0 - Intro" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Section G - CI_CD" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Section K - Migration" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Section H - Spark Optimization" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Section S - Cloud Map" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Section F - Databricks Azure" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1032,7 +1025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1050,144 +1043,168 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lakehouse | Delta Lake basics</t>
+          <t>CI/CD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Delta provides ACID, schema enforcement, and time travel on cloud storage. This enables reliable batch and streaming.</t>
+          <t>CDP: Bitbucket/Jenkins/RLM; Azure: Azure DevOps/GitHub; AWS: CodeBuild/CodeDeploy/CodePipeline; GCP: Cloud Build/Cloud Deploy.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lakehouse | Medallion architecture</t>
+          <t>Data Warehouse</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Explain Bronze for raw, Silver for cleaned, Gold for curated. This improves lineage and reusability.</t>
+          <t>CDP: Hive/Impala; Azure: Synapse; AWS: Redshift; GCP: BigQuery.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lakehouse | Auto Loader</t>
+          <t>Data Integration</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Incremental ingestion with schema inference and evolution. Use for scalable file discovery.</t>
+          <t>CDP: PySpark/NiFi/Sqoop; Azure: Data Factory; AWS: Glue/Data Pipeline; GCP: Data Fusion.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lakehouse | Delta Live Tables</t>
+          <t>Messaging</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Managed pipelines with declarative transformations and built-in quality checks. Useful for standard ETL.</t>
+          <t>CDP: JMS/Kafka; Azure: Service Bus/Event Hubs; AWS: Kinesis/SNS/SQS; GCP: Pub/Sub.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Compute | Cluster types</t>
+          <t>Workflow Orchestration</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>All-purpose for dev, job clusters for production. Job clusters reduce cost and improve isolation.</t>
+          <t>CDP: Oozie/Autosys/Airflow; Azure: Data Factory/Logic Apps; AWS: Step Functions/Glue Workflows; GCP: Composer.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Compute | Photon engine</t>
+          <t>Document DB</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Vectorized engine for faster SQL and Delta queries. Highlight when performance gains are most visible.</t>
+          <t>CDP: N/A or HBase; Azure: Cosmos DB; AWS: DocumentDB; GCP: Firestore.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Compute | Caching strategy</t>
+          <t>NoSQL (Key/Value)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cache reused DataFrames and unpersist after use. Avoid caching large single-use datasets.</t>
+          <t>CDP: HBase; Azure: Cosmos DB; AWS: DynamoDB; GCP: Bigtable.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Compute | OPTIMIZE and Z-ORDER</t>
+          <t>RDBMS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Compact small files and improve data skipping. Emphasize selective query performance.</t>
+          <t>CDP: Hive/Impala/Oracle; Azure: Azure SQL Database; AWS: Aurora/RDS; GCP: Cloud SQL.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Governance | Unity Catalog</t>
+          <t>Storage Transfer</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Centralized permissions, data discovery, and lineage. Enforce access by groups and domains.</t>
+          <t>CDP: DistCp/NiFi; Azure: Data Factory/Storage Mover; AWS: Storage Gateway/DataSync; GCP: Storage Transfer Service.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Governance | Secrets management</t>
+          <t>Network Connectivity</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Use secret scopes for credentials and rotate regularly. Avoid hard-coding secrets in notebooks.</t>
+          <t>CDP: Knox/SDX; Azure: VPN Gateway; AWS: VPN; GCP: Cloud VPN.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Governance | Repos and CI/CD</t>
+          <t>Audit Logging</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Git-backed repos allow code review and promotion. Automate deployments via pipelines.</t>
+          <t>CDP: Ranger Audit/Cloudera Navigator; Azure: Monitor/Audit Logs; AWS: CloudTrail; GCP: Cloud Audit Logs.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MLOps | MLflow basics</t>
+          <t>Key Management</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Track experiments, log metrics, and manage model registry. Enables reproducible ML workflows.</t>
+          <t>CDP: CyberArk/Ranger KMS; Azure: Key Vault; AWS: KMS; GCP: Cloud KMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Identity Management</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CDP: LDAP/Sentry/Ranger; Azure: Active Directory; AWS: IAM; GCP: Cloud IAM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CDP: HDFS; Azure: ADLS Gen2; AWS: S3; GCP: Cloud Storage.</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1220,1838 +1237,744 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Map CDP to Azure services</t>
+          <t>Databricks | What is a Lakehouse?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Map HDFS to ADLS, Hive to Delta/Synapse, Oozie to ADF/Workflows.</t>
+          <t>A Lakehouse combines data lake storage with warehouse governance and performance. In Databricks, Delta provides ACID, schema enforcement, and time travel to make it reliable for analytics.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Migrate Hive to Delta</t>
+          <t>Databricks | Delta Lake key benefits</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Convert schemas and data, validate, then optimize Delta tables.</t>
+          <t>Delta adds ACID transactions, schema enforcement, time travel, and scalable metadata. It prevents data corruption and simplifies incremental processing.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Migrate Sqoop to ADF/Databricks</t>
+          <t>Databricks | Medallion architecture</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Use ADF copy or Auto Loader for ingestion.</t>
+          <t>Bronze stores raw, Silver cleansed, Gold curated. This structure improves lineage, reusability, and controlled access for BI.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Migrate Oozie to ADF/Airflow</t>
+          <t>Databricks | Auto Loader use cases</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Translate workflows into pipelines or DAGs with triggers.</t>
+          <t>Use Auto Loader for incremental file ingestion at scale with schema evolution. It efficiently detects new files without heavy directory listing.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Migrate HDFS to ADLS Gen2</t>
+          <t>Databricks | Delta Live Tables (DLT)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Use DistCp or ADF; preserve ACLs and validate checksums.</t>
+          <t>DLT enables declarative ETL with built-in quality checks and lineage. It reduces boilerplate and standardizes pipelines.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Security and governance mapping</t>
+          <t>Databricks | Unity Catalog value</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Map Ranger/Sentry policies to Unity Catalog and Azure AD.</t>
+          <t>Unity Catalog centralizes permissions, data discovery, and lineage across workspaces. It enables consistent governance and auditability.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Performance tuning differences</t>
+          <t>Databricks | Photon engine</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tune partitions, caching, and clusters for Databricks.</t>
+          <t>Photon is a vectorized execution engine that speeds up SQL and Delta workloads. It is best for large scans and BI queries.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Common migration pitfalls</t>
+          <t>Databricks | Jobs vs All-purpose clusters</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Schema drift, small files, missing validation, or data loss.</t>
+          <t>Jobs clusters are ephemeral and cost-efficient for production. All-purpose clusters are interactive for development and exploration.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Testing and validation strategy</t>
+          <t>Databricks | Cluster sizing approach</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Row counts, aggregates, sampling, and reconciliation.</t>
+          <t>Start with 4-8 cores per executor and scale based on stage metrics. Use autoscaling for variable workloads and keep partitions balanced.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Cutover planning</t>
+          <t>Databricks | OPTIMIZE and Z-ORDER</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Parallel run, freeze window, and backout plan.</t>
+          <t>OPTIMIZE compacts small files; Z-ORDER co-locates data to improve data skipping. Use for selective query performance.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rollback planning</t>
+          <t>Databricks | VACUUM</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Keep legacy pipelines and data snapshots for quick revert.</t>
+          <t>VACUUM removes obsolete files and reduces metadata overhead. Coordinate with retention policies to avoid accidental data loss.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>On-prem to Databricks strategy</t>
+          <t>Databricks | Delta MERGE use case</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Assess, migrate data, refactor jobs, validate, cutover.</t>
+          <t>MERGE supports upserts and SCD patterns. It simplifies CDC ingestion by handling inserts, updates, and deletes in one statement.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hive to Delta conversion steps</t>
+          <t>Databricks | CDF (Change Data Feed)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Create Delta, backfill, validate, and optimize.</t>
+          <t>CDF exposes row-level changes for incremental processing. It reduces full-table scans and speeds downstream pipelines.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sqoop to Auto Loader/ADF</t>
+          <t>Databricks | Repos and CI/CD</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Replace batch loads with incremental ingestion.</t>
+          <t>Repos integrate Git for version control. Use CI/CD to test, deploy, and promote notebooks and jobs across environments.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Oozie to Databricks Workflows</t>
+          <t>Databricks | Secrets management</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Map actions to tasks and coordinators to schedules.</t>
+          <t>Store secrets in secret scopes and access via dbutils. Never hard-code credentials in notebooks or configs.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Parallel run strategy</t>
+          <t>Databricks | MLflow basics</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Run old and new pipelines in parallel for multiple cycles.</t>
+          <t>MLflow tracks experiments, metrics, and models. It improves reproducibility and manages model registry lifecycle.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Post-migration validation</t>
+          <t>Databricks | SQL Warehouses</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Compare counts, checksums, and business KPIs.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Batch/Lakehouse | Batch ETL design</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Describe source ingestion, staging, transforms, and curated outputs. Emphasize idempotency and partitioning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Batch/Lakehouse | Lakehouse architecture</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Combine data lake storage with warehouse governance. Use Bronze/Silver/Gold and Delta for ACID.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Batch/Lakehouse | Data modeling and grain</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Define grain before dimensions and facts. This prevents aggregation errors later.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Batch/Lakehouse | Partitioning strategy</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Partition by high-cardinality keys or time for pruning. Avoid over-partitioning small files.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Streaming | Real-time pipeline</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Use Structured Streaming with checkpoints and watermarking. Handle late data and exactly-once semantics.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Streaming | Lambda vs Kappa</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Lambda uses batch + stream; Kappa uses stream-only. Pick based on operational complexity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Streaming | CDC design</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Capture changes, dedupe with windows, and MERGE into targets. Maintain audit columns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Streaming | Backpressure handling</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Use rate limits and autoscaling. Monitor lag and tune micro-batch intervals.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Governance | Data quality framework</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Rule-driven checks with quarantine and audit logs. Fail fast on critical rules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Governance | Lineage and catalog</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Register schemas, owners, and lineage for impact analysis. Improves compliance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Governance | High availability</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Use multi-AZ storage, retries, and failover clusters. Design for graceful degradation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Governance | Cost optimization</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Use incremental loads, autoscaling, and right-sized clusters. Optimize file sizes to reduce scan cost.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Design | Job types</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Notebook, Python, JAR, and SQL tasks are supported. Choose based on codebase and runtime needs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Design | Job clusters vs all-purpose</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Job clusters are ephemeral and cost-efficient; all-purpose are interactive for development.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Design | Task orchestration</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Use task dependencies for DAG-style execution. Keep tasks small and idempotent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Design | Parameters and widgets</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Pass parameters via job inputs or widgets. This enables reusable pipelines.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ops | Scheduling</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Use cron or periodic schedules and align to SLAs. Avoid overlapping runs when not supported.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Ops | Retry and timeout strategy</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Set retries with backoff and timeouts per task. Fail fast on non-retriable errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ops | Monitoring and alerting</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Use job notifications, logs, and dashboards. Route alerts to on-call channels.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Ops | Environment separation</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Separate dev/test/prod with configs and permissions. Use workspace or catalog isolation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Security | Secrets in jobs</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Store credentials in secret scopes and reference them securely. Never embed secrets in code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Security | Service principals</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Use service principals for automated jobs. Grant least-privilege access.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Deployment | CI/CD for jobs</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Automate job creation and updates via pipelines. Keep job configs in version control.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Deployment | Rollback strategy</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Revert job config and code to last stable version. Use Delta time travel if needed.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Leadership | Tell me about yourself</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Provide a 60-second summary of experience, impact, and current focus. End with why the role fits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Leadership | Biggest project you led</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Highlight scope, stakeholders, and metrics. Focus on outcomes and lessons learned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Leadership | Conflict with stakeholder</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Explain the disagreement, how you aligned on priorities, and the compromise achieved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Execution | Production incident</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Use STAR: what broke, how you mitigated, and what you fixed permanently.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Execution | Handling tight deadlines</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Describe prioritization, scope reduction, and communication cadence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Execution | Process improvement</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Show how you automated a bottleneck and quantify the time saved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Growth | Weakness question</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Share a real weakness and the steps you took to improve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Growth | Failure you learned from</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Describe the failure, impact, and what you changed afterward.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Growth | Mentoring juniors</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Explain how you pair, review code, and give ownership with guidance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Leadership | Leadership style</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Describe how you balance autonomy, accountability, and support.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Execution | Managing priorities</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Use impact vs effort and align with business goals.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Leadership | Cross-team collaboration</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Show how you coordinate dependencies and keep decisions documented.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ingestion | Batch pipeline diagram</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Show sources, ingestion, staging, and curated layers. Emphasize partitioning and error handling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ingestion | Streaming pipeline diagram</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Show event source, streaming ingestion, checkpoints, and Delta sinks. Mention watermarking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Processing | Lakehouse layers</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Visualize Bronze/Silver/Gold with Delta and governance. Explain how data moves across layers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Processing | Serving layer</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Show BI or API access on Gold tables. Mention caching or SQL warehouses.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>DevOps | CI/CD flow</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Diagram source control, build/test, and deployment stages. Include approval gates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>DevOps | Monitoring layer</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Include logs, metrics, and alerting for pipelines. Show how failures are triaged.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Migration | Cutover diagram</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Show parallel runs, validation checks, and final cutover. Include rollback path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Migration | Data validation steps</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Show row counts, checksums, and business KPI reconciliation.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Databricks | What is Delta Lake?</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Delta adds ACID transactions, schema enforcement, and time travel on cloud storage. It reduces data corruption and enables reliable pipelines.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Databricks | When to use Auto Loader?</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Use Auto Loader for incremental file ingestion at scale. It handles schema evolution and efficient file discovery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Databricks | Explain Unity Catalog</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Unity Catalog centralizes governance for data, permissions, and lineage. It enables consistent access controls across workspaces.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Databricks | What is Photon?</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Photon is a vectorized execution engine for faster SQL and Delta workloads. It helps with BI and large scans.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Databricks | Delta OPTIMIZE vs VACUUM</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>OPTIMIZE compacts small files for faster reads. VACUUM removes obsolete files to reduce storage and metadata.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Spark | RDD vs DataFrame vs Dataset</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>RDD is low-level and flexible; DataFrame is optimized and schema-based; Dataset adds types in Scala/Java.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Spark | What causes shuffles?</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Wide transformations like join, groupBy, and distinct trigger shuffles. They are expensive and should be minimized.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Spark | How to handle skew?</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Use salting, broadcast joins, or range partitioning. Validate improvements in Spark UI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Spark | Explain AQE</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Adaptive Query Execution adjusts joins, skew, and partitions at runtime. It improves stability and performance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Spark | Cache vs persist</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Cache uses memory by default; persist allows different storage levels. Use when datasets are reused.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>SQL | Difference between RANK and DENSE_RANK</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RANK leaves gaps after ties; DENSE_RANK does not. Choose based on reporting needs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>SQL | Find duplicates</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>GROUP BY columns and HAVING COUNT(*) &gt; 1 identifies duplicates. Join back to get full rows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>SQL | Nth highest salary</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Use DENSE_RANK over salary DESC and filter rnk = N. Handles ties correctly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>SQL | Window functions use cases</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Running totals, ranking, and lag/lead comparisons. They avoid complex self-joins.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SQL | How to compare two tables</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Use FULL OUTER JOIN or EXCEPT/UNION to detect mismatches. Validate on key columns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Databricks | CDC pipeline design</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Ingest changes, dedupe by key/time, then MERGE into Delta. Maintain audit columns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Spark | Optimize slow job</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Profile stages, fix skew, prune columns, tune partitions, and cache reused data.</t>
+          <t>Use SQL Warehouses for BI and ad-hoc analytics. Choose serverless or pro based on concurrency and cost.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Governance | How do you handle PII?</t>
+          <t>Databricks | When to use notebooks vs jobs</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mask or tokenize sensitive fields and restrict access with RBAC. Log access for audits.</t>
+          <t>Use notebooks for exploration and iterative development; use jobs for scheduled, production-grade workflows.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Reliability | How to rollback bad release?</t>
+          <t>Databricks | Delta vs Parquet</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Revert code, restore Delta tables with time travel, and rerun affected jobs.</t>
+          <t>Delta is Parquet plus transaction log, enabling ACID and schema enforcement. Choose Delta for reliable analytics pipelines.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Modeling | Fact vs dimension</t>
+          <t>Databricks | Caching strategy</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Facts store measures and foreign keys; dimensions store descriptive attributes. Grain is critical.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B44"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Driver, executors, cluster manager</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Driver schedules work; executors run tasks; manager allocates resources.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>RDD vs DataFrame vs Dataset</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RDD is low-level; DataFrame is optimized; Dataset is typed (Scala/Java).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Lazy evaluation</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Transforms build a DAG; actions trigger execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Transformations vs actions</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Transformations create lineage; actions materialize results.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Narrow vs wide transformations</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Narrow avoids shuffle; wide causes shuffle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Catalyst optimizer</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Optimizes logical and physical plans for SQL/DataFrames.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Tungsten engine</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Uses codegen and binary processing for performance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Shuffle mechanics</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Shuffle moves data across partitions and is expensive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Broadcast joins</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Broadcast small tables to avoid shuffle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Broadcast hint</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Force broadcast when auto-broadcast does not trigger.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Caching and persisting</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Cache reused DataFrames; unpersist when done.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Partitioning strategy</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Partition by high-cardinality keys for parallelism, low-cardinality for pruning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Repartition vs coalesce</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Repartition balances with shuffle; coalesce reduces partitions without shuffle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>AQE</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Adaptive Query Execution tunes joins, skew, and partitions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Shuffle partitions tuning</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Adjust spark.sql.shuffle.partitions to cluster size.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Skew handling</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Use salting, range partitioning, or broadcast to fix skew.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Predicate pushdown</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Push filters to source to reduce scan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Column pruning</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Select only required columns to save memory.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Avoid Python UDFs</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Prefer built-in functions or pandas UDFs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Avoid wide transformations</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Filter early and pre-aggregate to reduce shuffles.</t>
+          <t>Cache reused datasets, but avoid caching large single-use tables. Always unpersist to free memory.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>mapPartitions vs map</t>
+          <t>Databricks | Explain AQE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Process batches per partition for efficiency.</t>
+          <t>Adaptive Query Execution optimizes joins, skew, and shuffle partitions at runtime. It improves stability on changing data volumes.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Avoid collect()</t>
+          <t>Azure | ADLS Gen2 as data lake</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Do not bring large data to driver.</t>
+          <t>ADLS Gen2 provides hierarchical namespace and POSIX ACLs. It is the primary storage layer for lakehouse patterns.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Avoid explode on large arrays</t>
+          <t>Azure | Databricks + ADLS integration</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Explode can cause huge shuffles; pre-filter arrays.</t>
+          <t>Mount ADLS via ABFS or use direct access with service principal. Ensure least-privilege access and token rotation.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Window functions</t>
+          <t>Azure | ADF orchestration with Databricks</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Partition wisely; window ops can shuffle.</t>
+          <t>ADF triggers notebooks, passes parameters, and controls dependencies. Use ADF for workflow orchestration and Databricks for compute.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>File size tuning</t>
+          <t>Azure | Azure Key Vault usage</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Target 128-512 MB files to avoid small-file overhead.</t>
+          <t>Store secrets, keys, and certificates in Key Vault. Integrate with Databricks secret scopes for secure access.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Delta OPTIMIZE</t>
+          <t>Azure | Azure AD integration</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Compact small files to improve reads.</t>
+          <t>Use Azure AD for authentication and group-based authorization. Align Unity Catalog permissions with AD groups.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Z-ORDER</t>
+          <t>Azure | VNet injection</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Co-locate data to improve selective query skipping.</t>
+          <t>Deploy Databricks in a VNet for secure networking and private access. Pair with Private Link for data sources.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Data skipping stats</t>
+          <t>Azure | Private Link for storage</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Delta stores min/max stats for pruning.</t>
+          <t>Private Link keeps data traffic on Microsoft backbone. It improves security and meets compliance requirements.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Bloom filters</t>
+          <t>Azure | Synapse vs Databricks</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Speed up selective joins and lookups.</t>
+          <t>Synapse is warehouse-centric; Databricks excels at Spark and ML. Choose based on workload mix and team skillset.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Delta MERGE</t>
+          <t>Azure | Data Factory vs Databricks Workflows</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Use MERGE for upserts and SCD handling.</t>
+          <t>ADF is best for cross-service orchestration; Workflows are better for Spark-native pipelines.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Delta CDF</t>
+          <t>Azure | Cost management approach</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Use Change Data Feed for incremental processing.</t>
+          <t>Use cluster policies, autoscaling, and job clusters. Track cost by workspace and use tags for chargeback.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Auto Loader</t>
+          <t>Design | End-to-end lakehouse pipeline</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Incremental ingestion with schema evolution.</t>
+          <t>Ingest to Bronze, cleanse to Silver, and aggregate to Gold. Use Delta for ACID, checkpoints for streaming, and audit tables for observability.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Auto-Optimize / Optimize Write</t>
+          <t>Design | CDC pipeline design</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Auto-compact files during writes.</t>
+          <t>Extract incremental changes, dedupe by key and timestamp, and MERGE into targets. Maintain audit columns and handle late-arriving data.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>VACUUM</t>
+          <t>Design | Data quality framework</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Remove obsolete files to reduce metadata and storage.</t>
+          <t>Define rules in metadata, apply checks in ETL, quarantine failures, and surface dashboards for monitoring.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Liquid clustering</t>
+          <t>Design | Streaming pipeline essentials</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Next-gen clustering for large Delta tables.</t>
+          <t>Use Structured Streaming with checkpoints, watermarking, and idempotent sinks. Monitor lag and tune micro-batch intervals.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Photon engine</t>
+          <t>Design | Schema evolution strategy</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Vectorized engine for faster SQL/Delta on Databricks.</t>
+          <t>Enforce schema on write and allow controlled evolution with audits. Protect downstream consumers from breaking changes.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Avoid cross joins</t>
+          <t>Design | Partitioning strategy</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cross joins explode data unless required.</t>
+          <t>Partition by time or high-cardinality keys for pruning. Avoid over-partitioning to reduce small files.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Incremental ETL</t>
+          <t>Design | Data modeling in lakehouse</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Process only changes to reduce cost and latency.</t>
+          <t>Define grain and keys before modeling facts and dimensions. Keep semantic layer aligned with BI needs.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Range partitioning for time-series</t>
+          <t>Design | Medallion vs Data Vault</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Partition by date for pruning and parallelism.</t>
+          <t>Medallion is layer-based for analytics; Data Vault is hub/satellite for auditability. Choose based on lineage and compliance needs.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Checkpointing</t>
+          <t>Operations | Monitoring strategy</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Break long lineage and improve stability.</t>
+          <t>Use job logs, Spark UI, and metrics dashboards. Set alerts on failures, SLA breaches, and lag.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Avoid repeated reads</t>
+          <t>Operations | Handling skew</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Cache or checkpoint to reuse datasets.</t>
+          <t>Detect skew via Spark UI and fix with salting, broadcast joins, or range partitioning.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Use explain()</t>
+          <t>Operations | Reducing shuffle</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Inspect plans to spot expensive stages.</t>
+          <t>Filter early, pre-aggregate, and partition on join keys. Avoid wide transformations when possible.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Cluster sizing and autoscaling</t>
+          <t>Operations | Small files problem</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Right-size executors and use autoscaling for peak loads.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CI/CD</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>CDP: Bitbucket/Jenkins/RLM; Azure: Azure DevOps/GitHub; AWS: CodeBuild/CodeDeploy/CodePipeline; GCP: Cloud Build/Cloud Deploy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Data Warehouse</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CDP: Hive/Impala; Azure: Synapse; AWS: Redshift; GCP: BigQuery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Data Integration</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>CDP: PySpark/NiFi/Sqoop; Azure: Data Factory; AWS: Glue/Data Pipeline; GCP: Data Fusion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Messaging</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>CDP: JMS/Kafka; Azure: Service Bus/Event Hubs; AWS: Kinesis/SNS/SQS; GCP: Pub/Sub.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Workflow Orchestration</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CDP: Oozie/Autosys/Airflow; Azure: Data Factory/Logic Apps; AWS: Step Functions/Glue Workflows; GCP: Composer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Document DB</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CDP: N/A or HBase; Azure: Cosmos DB; AWS: DocumentDB; GCP: Firestore.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>NoSQL (Key/Value)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>CDP: HBase; Azure: Cosmos DB; AWS: DynamoDB; GCP: Bigtable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>RDBMS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CDP: Hive/Impala/Oracle; Azure: Azure SQL Database; AWS: Aurora/RDS; GCP: Cloud SQL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Storage Transfer</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CDP: DistCp/NiFi; Azure: Data Factory/Storage Mover; AWS: Storage Gateway/DataSync; GCP: Storage Transfer Service.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Network Connectivity</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CDP: Knox/SDX; Azure: VPN Gateway; AWS: VPN; GCP: Cloud VPN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Audit Logging</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>CDP: Ranger Audit/Cloudera Navigator; Azure: Monitor/Audit Logs; AWS: CloudTrail; GCP: Cloud Audit Logs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Key Management</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CDP: CyberArk/Ranger KMS; Azure: Key Vault; AWS: KMS; GCP: Cloud KMS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Identity Management</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>CDP: LDAP/Sentry/Ranger; Azure: Active Directory; AWS: IAM; GCP: Cloud IAM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Storage</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>CDP: HDFS; Azure: ADLS Gen2; AWS: S3; GCP: Cloud Storage.</t>
+          <t>Compact files via OPTIMIZE, auto-compact, or coalesce on write. Target 128-512 MB per file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Operations | Debugging failed jobs</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Check driver/executor logs, inspect input anomalies, and reproduce with small samples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Operations | Incident response at 2 AM</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Triage impact, communicate status, rerun with backfill, and add alerts to prevent recurrence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Jobs | Parameterization best practices</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Use widgets or job parameters for environments and dates. Keep defaults safe and validate inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Jobs | Retry and timeout strategy</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Set retries with backoff for transient issues and strict timeouts for runaway tasks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Jobs | Promotion across environments</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Use CI/CD to promote tested artifacts. Keep environment configs in versioned files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Jobs | Alerting and SLAs</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Send alerts to on-call channels and define clear SLAs. Use run metrics to track reliability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Jobs | Secret handling in jobs</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Access credentials via secret scopes or Key Vault integration. Avoid logging secrets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Behavioral | Tell me about yourself</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Summarize experience, impact, and why Databricks/Azure aligns with your goals. Keep it under 60 seconds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Behavioral | Biggest project led</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Highlight scope, stakeholders, and measurable outcomes. Emphasize leadership and technical decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Behavioral | Conflict with stakeholder</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Describe how you aligned priorities, delivered a phased solution, and protected quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Behavioral | Failure and learning</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Explain the failure, the root cause, and the process improvement you implemented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Behavioral | Mentoring juniors</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Discuss pairing, code reviews, and gradual ownership. Show how you measure growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Mock QA | RDD vs DataFrame vs Dataset</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>RDD is low-level and untyped; DataFrame is optimized; Dataset adds types in Scala/Java. Prefer DataFrames in Python.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Mock QA | When to broadcast join</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Broadcast when one side is small enough to fit in memory. This avoids shuffle and speeds joins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Mock QA | Delta time travel</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Time travel lets you query previous versions for recovery or audit. It is key for rollback scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Mock QA | Z-ORDER purpose</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Z-ORDER clusters data to improve skipping for selective queries. Use after OPTIMIZE on large tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Mock QA | Spark shuffle triggers</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Wide operations like join, groupBy, distinct, and repartition trigger shuffles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Mock QA | How to compare two tables</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Use FULL OUTER JOIN or EXCEPT to find mismatches. Always compare on business keys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Mock QA | How to handle PII</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Mask or tokenize fields, enforce RBAC, and audit access. Align with compliance policies.</t>
         </is>
       </c>
     </row>
@@ -4521,20 +3444,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
@@ -4543,144 +3462,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Platform | Warehouse choices</t>
+          <t>Profile summary</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Explain trade-offs: Redshift and Synapse are warehouse-first; BigQuery is serverless and scales per query. Tie selection to workload, cost model, and latency needs.</t>
+          <t>13+ years in data engineering across CDP, Databricks, ETL, governance.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Platform | Storage layer</t>
+          <t>Core skills</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Compare ADLS, S3, GCS for durability, cost, and integration. Mention partitioning strategy and lifecycle policies.</t>
+          <t>Python, SQL, PySpark, data modeling, data quality, Agile.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Platform | Databricks vs native warehouse</t>
+          <t>Cloud platforms</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Choose Databricks for Spark/Delta and ML workloads; choose native warehouse for pure BI analytics. Highlight interoperability when both are used.</t>
+          <t>Cloudera CDP/CDH, Azure, AWS, GCP, Databricks.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Integration | ETL tool selection</t>
+          <t>ETL tools</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ADF, Glue, and Data Fusion all orchestrate ingestion; choose based on cloud footprint and connector needs. Note cost, integration, and monitoring features.</t>
+          <t>ADF, Databricks, SSIS, Informatica.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Integration | Orchestration strategy</t>
+          <t>Big data technologies</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Airflow provides portable DAGs; ADF provides managed pipelines in Azure. Discuss retries, SLA alerts, and dependency handling.</t>
+          <t>Spark, Hadoop, HDFS, Hive, Sqoop, Kafka.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Integration | Event streaming</t>
+          <t>CI/CD and automation</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kafka/Kinesis/PubSub differ by managed depth and ecosystem. Emphasize ordering, partitions, and consumer lag monitoring.</t>
+          <t>Jenkins, RLM DevOps, Git, GitHub, Bitbucket.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Integration | CI/CD for data pipelines</t>
+          <t>Migration experience</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Use Git-based workflows and automated tests for notebooks and SQL. Promote artifacts across environments with approvals.</t>
+          <t>Cloudera to Azure Databricks lakehouse migrations.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Governance | IAM and RBAC</t>
+          <t>REST API integration</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Use least privilege with service principals and group-based access. Tie to Unity Catalog or cloud IAM policies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Governance | Data catalog and lineage</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Use catalog for schema ownership and lineage for auditability. This improves compliance and impact analysis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Governance | PII handling</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Apply masking, encryption, and access controls. Audit access and enforce data retention policies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Governance | Key management</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Use KMS/Key Vault and rotate secrets. Separate keys per environment for risk isolation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Governance | Data quality checks</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Implement null, range, and referential integrity checks in pipelines. Fail fast and quarantine bad records.</t>
+          <t>Python REST APIs for ingestion and conversion.</t>
         </is>
       </c>
     </row>
@@ -4695,7 +3566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4713,96 +3584,144 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Profile summary</t>
+          <t>Git clone/pull/push/fetch</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>13+ years in data engineering across CDP, Databricks, ETL, governance.</t>
+          <t>Clone repo, fetch updates, pull merge, push commits.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Core skills</t>
+          <t>Git branching strategy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Python, SQL, PySpark, data modeling, data quality, Agile.</t>
+          <t>Use feature branches and PRs; keep main stable.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cloud platforms</t>
+          <t>Git merge vs rebase</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cloudera CDP/CDH, Azure, AWS, GCP, Databricks.</t>
+          <t>Merge preserves history; rebase creates linear history.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ETL tools</t>
+          <t>Git stash</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ADF, Databricks, SSIS, Informatica.</t>
+          <t>Temporarily save uncommitted changes.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Big data technologies</t>
+          <t>Git revert vs reset</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Spark, Hadoop, HDFS, Hive, Sqoop, Kafka.</t>
+          <t>Revert adds a new commit; reset rewrites history.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CI/CD and automation</t>
+          <t>Jenkins pipeline stages</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jenkins, RLM DevOps, Git, GitHub, Bitbucket.</t>
+          <t>Checkout, build, test, package, deploy.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Migration experience</t>
+          <t>Build-Test-Deploy flow</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cloudera to Azure Databricks lakehouse migrations.</t>
+          <t>Automate compile, validate, release steps.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>REST API integration</t>
+          <t>CI triggers (webhooks)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Python REST APIs for ingestion and conversion.</t>
+          <t>Start pipeline on push or PR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CD deployment strategies</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Blue/green, canary, rolling, or shadow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rollback strategy</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Keep versioned artifacts and revert quickly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Versioning and tagging</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Use semantic versioning and Git tags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Code review best practices</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Small PRs, tests, style, and design checks.</t>
         </is>
       </c>
     </row>
@@ -4817,7 +3736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4835,144 +3754,204 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Git clone/pull/push/fetch</t>
+          <t>Map CDP to Azure services</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Clone repo, fetch updates, pull merge, push commits.</t>
+          <t>Map HDFS to ADLS, Hive to Delta/Synapse, Oozie to ADF/Workflows.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Git branching strategy</t>
+          <t>Migrate Hive to Delta</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Use feature branches and PRs; keep main stable.</t>
+          <t>Convert schemas and data, validate, then optimize Delta tables.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Git merge vs rebase</t>
+          <t>Migrate Sqoop to ADF/Databricks</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Merge preserves history; rebase creates linear history.</t>
+          <t>Use ADF copy or Auto Loader for ingestion.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Git stash</t>
+          <t>Migrate Oozie to ADF/Airflow</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Temporarily save uncommitted changes.</t>
+          <t>Translate workflows into pipelines or DAGs with triggers.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Git revert vs reset</t>
+          <t>Migrate HDFS to ADLS Gen2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Revert adds a new commit; reset rewrites history.</t>
+          <t>Use DistCp or ADF; preserve ACLs and validate checksums.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jenkins pipeline stages</t>
+          <t>Security and governance mapping</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Checkout, build, test, package, deploy.</t>
+          <t>Map Ranger/Sentry policies to Unity Catalog and Azure AD.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Build-Test-Deploy flow</t>
+          <t>Performance tuning differences</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Automate compile, validate, release steps.</t>
+          <t>Tune partitions, caching, and clusters for Databricks.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CI triggers (webhooks)</t>
+          <t>Common migration pitfalls</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Start pipeline on push or PR.</t>
+          <t>Schema drift, small files, missing validation, or data loss.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CD deployment strategies</t>
+          <t>Testing and validation strategy</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Blue/green, canary, rolling, or shadow.</t>
+          <t>Row counts, aggregates, sampling, and reconciliation.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rollback strategy</t>
+          <t>Cutover planning</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Keep versioned artifacts and revert quickly.</t>
+          <t>Parallel run, freeze window, and backout plan.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Versioning and tagging</t>
+          <t>Rollback planning</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Use semantic versioning and Git tags.</t>
+          <t>Keep legacy pipelines and data snapshots for quick revert.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Code review best practices</t>
+          <t>On-prem to Databricks strategy</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Small PRs, tests, style, and design checks.</t>
+          <t>Assess, migrate data, refactor jobs, validate, cutover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hive to Delta conversion steps</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Create Delta, backfill, validate, and optimize.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sqoop to Auto Loader/ADF</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Replace batch loads with incremental ingestion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Oozie to Databricks Workflows</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Map actions to tasks and coordinators to schedules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Parallel run strategy</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Run old and new pipelines in parallel for multiple cycles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Post-migration validation</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Compare counts, checksums, and business KPIs.</t>
         </is>
       </c>
     </row>
@@ -4987,7 +3966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5005,180 +3984,516 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Architecture | End-to-end ADF + Databricks pipeline</t>
+          <t>Driver, executors, cluster manager</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Describe ingestion with ADF, processing in Databricks, and Delta storage in Bronze/Silver/Gold. Emphasize idempotency and monitoring.</t>
+          <t>Driver schedules work; executors run tasks; manager allocates resources.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Architecture | Lakehouse design</t>
+          <t>RDD vs DataFrame vs Dataset</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Use ADLS + Delta + Unity Catalog. Explain how governance and performance are balanced in the Gold layer.</t>
+          <t>RDD is low-level; DataFrame is optimized; Dataset is typed (Scala/Java).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Architecture | CDC ingestion</t>
+          <t>Lazy evaluation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Capture changes, dedupe by key and timestamp, then MERGE into targets. Highlight late-arriving data handling.</t>
+          <t>Transforms build a DAG; actions trigger execution.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Architecture | Schema evolution</t>
+          <t>Transformations vs actions</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Enforce schema on write and allow controlled evolution with audits. Protect downstream consumers from breaking changes.</t>
+          <t>Transformations create lineage; actions materialize results.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Architecture | Migration plan</t>
+          <t>Narrow vs wide transformations</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Map CDP services to Azure, migrate data, refactor jobs, validate, then cutover. Use parallel runs to reduce risk.</t>
+          <t>Narrow avoids shuffle; wide causes shuffle.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Performance | Reduce 3-hour Spark job</t>
+          <t>Catalyst optimizer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Profile stages, fix skew, prune columns, and tune partitions. Show before/after metrics to prove improvement.</t>
+          <t>Optimizes logical and physical plans for SQL/DataFrames.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Performance | Handle data skew</t>
+          <t>Tungsten engine</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Use salting, broadcast joins, or range partitioning. Validate skew reduction in Spark UI.</t>
+          <t>Uses codegen and binary processing for performance.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Performance | Reduce shuffles</t>
+          <t>Shuffle mechanics</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Avoid wide transformations and pre-aggregate early. Partition by join keys to minimize shuffle volume.</t>
+          <t>Shuffle moves data across partitions and is expensive.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Performance | Cost optimization</t>
+          <t>Broadcast joins</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Right-size clusters, use autoscaling, and optimize file sizes. Reduce recompute via caching and incremental loads.</t>
+          <t>Broadcast small tables to avoid shuffle.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Reliability | Debug failing Spark jobs</t>
+          <t>Broadcast hint</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Check driver/executor logs and the Spark UI. Reproduce with small samples and add data quality checks.</t>
+          <t>Force broadcast when auto-broadcast does not trigger.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reliability | Recover Delta tables</t>
+          <t>Caching and persisting</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Use time travel or restore from checkpoints. Explain how you validate data consistency post-recovery.</t>
+          <t>Cache reused DataFrames; unpersist when done.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Reliability | 2 AM pipeline failure</t>
+          <t>Partitioning strategy</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Triage quickly, communicate impact, rerun with backfill, and add alerts to prevent repeat issues.</t>
+          <t>Partition by high-cardinality keys for parallelism, low-cardinality for pruning.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Leadership | Mentor junior engineers</t>
+          <t>Repartition vs coalesce</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Use pairing, code reviews, and clear ownership. Tie feedback to measurable growth milestones.</t>
+          <t>Repartition balances with shuffle; coalesce reduces partitions without shuffle.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Leadership | Conflicting requirements</t>
+          <t>AQE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Align on priorities with stakeholders and deliver in phases. Provide a clear trade-off summary.</t>
+          <t>Adaptive Query Execution tunes joins, skew, and partitions.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Leadership | Communicate delays</t>
+          <t>Shuffle partitions tuning</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Share root cause, new timeline, and mitigation steps. Keep stakeholders updated until resolution.</t>
+          <t>Adjust spark.sql.shuffle.partitions to cluster size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Skew handling</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Use salting, range partitioning, or broadcast to fix skew.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Predicate pushdown</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Push filters to source to reduce scan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Column pruning</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Select only required columns to save memory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Avoid Python UDFs</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Prefer built-in functions or pandas UDFs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Avoid wide transformations</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Filter early and pre-aggregate to reduce shuffles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>mapPartitions vs map</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Process batches per partition for efficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Avoid collect()</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Do not bring large data to driver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Avoid explode on large arrays</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Explode can cause huge shuffles; pre-filter arrays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Window functions</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Partition wisely; window ops can shuffle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>File size tuning</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Target 128-512 MB files to avoid small-file overhead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Delta OPTIMIZE</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Compact small files to improve reads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Z-ORDER</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Co-locate data to improve selective query skipping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Data skipping stats</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Delta stores min/max stats for pruning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Bloom filters</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Speed up selective joins and lookups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Delta MERGE</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Use MERGE for upserts and SCD handling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Delta CDF</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Use Change Data Feed for incremental processing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Auto Loader</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Incremental ingestion with schema evolution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Auto-Optimize / Optimize Write</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Auto-compact files during writes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>VACUUM</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Remove obsolete files to reduce metadata and storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Liquid clustering</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Next-gen clustering for large Delta tables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Photon engine</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Vectorized engine for faster SQL/Delta on Databricks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Avoid cross joins</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Cross joins explode data unless required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Incremental ETL</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Process only changes to reduce cost and latency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Range partitioning for time-series</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Partition by date for pruning and parallelism.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Checkpointing</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Break long lineage and improve stability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Avoid repeated reads</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Cache or checkpoint to reuse datasets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Use explain()</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Inspect plans to spot expensive stages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Cluster sizing and autoscaling</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Right-size executors and use autoscaling for peak loads.</t>
         </is>
       </c>
     </row>

</xml_diff>